<commit_message>
Update NY gaming data - Thu Jul 23 15:35:37 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -213,10 +213,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,15 +237,12 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -259,12 +253,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -771,53 +759,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>7/5/2026</t>
+          <t>7/12/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>198331851</v>
+        <v>165737601</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>13762042</v>
+        <v>23467231</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.06938896566845433</v>
+        <v>0.1415926793823931</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>187715921</v>
+        <v>162520980</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>13578971</v>
+        <v>24960939</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.07233787591197445</v>
+        <v>0.1535859493340491</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>39155250</v>
+        <v>34868855</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>2644188</v>
+        <v>4459574</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.06753086750818856</v>
+        <v>0.1278956249065248</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>62287631</v>
+        <v>51411108</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>3223781</v>
+        <v>7470125</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.05175635913974638</v>
+        <v>0.1453017701933209</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>548797512</v>
+        <v>464461727</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>36510807</v>
+        <v>65981611</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.06652874002096423</v>
+        <v>0.1420603833736337</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -828,264 +816,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+48%</t>
+          <t>+35%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>+2%</t>
+          <t>+87%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>-319bps</t>
+          <t>+391bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+57%</t>
+          <t>+45%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>+1%</t>
+          <t>+65%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>-407bps</t>
+          <t>+189bps</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>+60%</t>
+          <t>+55%</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>+20%</t>
+          <t>+161%</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>-223bps</t>
+          <t>+520bps</t>
         </is>
       </c>
       <c r="K4" s="13" t="inlineStr">
         <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="L4" s="16" t="inlineStr">
-        <is>
-          <t>-9%</t>
+          <t>+68%</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>+161%</t>
         </is>
       </c>
       <c r="M4" s="15" t="inlineStr">
         <is>
-          <t>-612bps</t>
+          <t>+519bps</t>
         </is>
       </c>
       <c r="N4" s="13" t="inlineStr">
         <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="O4" s="16" t="inlineStr">
-        <is>
-          <t>-4%</t>
+          <t>+41%</t>
+        </is>
+      </c>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>+89%</t>
         </is>
       </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
-          <t>-410bps</t>
+          <t>+356bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>6/28/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="n">
-        <v>187265340</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>20773685</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.1109318200581058</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>178427790</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>25667736</v>
-      </c>
-      <c r="G5" s="20" t="n">
-        <v>0.1438550351377439</v>
-      </c>
-      <c r="H5" s="18" t="n">
-        <v>34322403</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>4555167</v>
-      </c>
-      <c r="J5" s="20" t="n">
-        <v>0.1327170186772762</v>
-      </c>
-      <c r="K5" s="18" t="n">
-        <v>59305990</v>
-      </c>
-      <c r="L5" s="19" t="n">
-        <v>5238538</v>
-      </c>
-      <c r="M5" s="20" t="n">
-        <v>0.08833067283760039</v>
-      </c>
-      <c r="N5" s="18" t="n">
-        <v>512508333</v>
-      </c>
-      <c r="O5" s="19" t="n">
-        <v>61849542</v>
-      </c>
-      <c r="P5" s="20" t="n">
-        <v>0.120680070971646</v>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>7/5/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>198331851</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>13762042</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0.06938896566845433</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>187715921</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>13578971</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>0.07233787591197445</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>39155250</v>
+      </c>
+      <c r="I5" s="18" t="n">
+        <v>2644188</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>0.06753086750818856</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>62287631</v>
+      </c>
+      <c r="L5" s="18" t="n">
+        <v>3223781</v>
+      </c>
+      <c r="M5" s="19" t="n">
+        <v>0.05175635913974638</v>
+      </c>
+      <c r="N5" s="17" t="n">
+        <v>548797512</v>
+      </c>
+      <c r="O5" s="18" t="n">
+        <v>36510807</v>
+      </c>
+      <c r="P5" s="19" t="n">
+        <v>0.06652874002096423</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>+306bps</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>+49%</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>+67%</t>
-        </is>
-      </c>
-      <c r="G6" s="24" t="inlineStr">
-        <is>
-          <t>+158bps</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="I6" s="23" t="inlineStr">
-        <is>
-          <t>+417%</t>
-        </is>
-      </c>
-      <c r="J6" s="24" t="inlineStr">
-        <is>
-          <t>+974bps</t>
-        </is>
-      </c>
-      <c r="K6" s="22" t="inlineStr">
-        <is>
-          <t>+73%</t>
-        </is>
-      </c>
-      <c r="L6" s="23" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="M6" s="24" t="inlineStr">
-        <is>
-          <t>+117bps</t>
-        </is>
-      </c>
-      <c r="N6" s="22" t="inlineStr">
-        <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="O6" s="23" t="inlineStr">
-        <is>
-          <t>+86%</t>
-        </is>
-      </c>
-      <c r="P6" s="24" t="inlineStr">
-        <is>
-          <t>+255bps</t>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>+2%</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>-319bps</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>+1%</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>-407bps</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>+60%</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>+20%</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>-223bps</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="inlineStr">
+        <is>
+          <t>+98%</t>
+        </is>
+      </c>
+      <c r="L6" s="24" t="inlineStr">
+        <is>
+          <t>-9%</t>
+        </is>
+      </c>
+      <c r="M6" s="23" t="inlineStr">
+        <is>
+          <t>-612bps</t>
+        </is>
+      </c>
+      <c r="N6" s="21" t="inlineStr">
+        <is>
+          <t>+55%</t>
+        </is>
+      </c>
+      <c r="O6" s="24" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="P6" s="23" t="inlineStr">
+        <is>
+          <t>-410bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>6/21/2026</t>
+          <t>6/28/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>196191527</v>
+        <v>187265340</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>15707056</v>
+        <v>20773685</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.08005980808743081</v>
+        <v>0.1109318200581058</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>197643614</v>
+        <v>178427790</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>24458285</v>
+        <v>25667736</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1237494321470968</v>
+        <v>0.1438550351377439</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>37762064</v>
+        <v>34322403</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>3330257</v>
+        <v>4555167</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.08819054488123319</v>
+        <v>0.1327170186772762</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>64128131</v>
+        <v>59305990</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>3055347</v>
+        <v>5238538</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.04764441053178362</v>
+        <v>0.08833067283760039</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>551320172</v>
+        <v>512508333</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>50756045</v>
+        <v>61849542</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.09206273881812545</v>
+        <v>0.120680070971646</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1096,345 +1084,345 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>+35%</t>
+          <t>+45%</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>+1%</t>
+          <t>+100%</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>-267bps</t>
+          <t>+306bps</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>+42%</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>-3%</t>
+          <t>+49%</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>+67%</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>-576bps</t>
+          <t>+158bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+30%</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>-25%</t>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>+417%</t>
         </is>
       </c>
       <c r="J8" s="15" t="inlineStr">
         <is>
-          <t>-649bps</t>
+          <t>+974bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>+71%</t>
-        </is>
-      </c>
-      <c r="L8" s="16" t="inlineStr">
-        <is>
-          <t>-39%</t>
+          <t>+73%</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>+100%</t>
         </is>
       </c>
       <c r="M8" s="15" t="inlineStr">
         <is>
-          <t>-867bps</t>
+          <t>+117bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="O8" s="16" t="inlineStr">
-        <is>
-          <t>-8%</t>
+          <t>+47%</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>+86%</t>
         </is>
       </c>
       <c r="P8" s="15" t="inlineStr">
         <is>
-          <t>-469bps</t>
+          <t>+255bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>6/14/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>195613214</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>-14033670</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>-0.07174193252609203</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>220845889</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>-22574161</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>-0.1022168042258645</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>44703354</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>-2481951</v>
-      </c>
-      <c r="J9" s="20" t="n">
-        <v>-0.05552046497450728</v>
-      </c>
-      <c r="K9" s="18" t="n">
-        <v>67325791</v>
-      </c>
-      <c r="L9" s="19" t="n">
-        <v>-5819762</v>
-      </c>
-      <c r="M9" s="20" t="n">
-        <v>-0.08644179167534771</v>
-      </c>
-      <c r="N9" s="18" t="n">
-        <v>587580124</v>
-      </c>
-      <c r="O9" s="19" t="n">
-        <v>-48515978</v>
-      </c>
-      <c r="P9" s="20" t="n">
-        <v>-0.08256912720213117</v>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>6/21/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>196191527</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>15707056</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.08005980808743081</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>197643614</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>24458285</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>0.1237494321470968</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>37762064</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>3330257</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0.08819054488123319</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <v>64128131</v>
+      </c>
+      <c r="L9" s="18" t="n">
+        <v>3055347</v>
+      </c>
+      <c r="M9" s="19" t="n">
+        <v>0.04764441053178362</v>
+      </c>
+      <c r="N9" s="17" t="n">
+        <v>551320172</v>
+      </c>
+      <c r="O9" s="18" t="n">
+        <v>50756045</v>
+      </c>
+      <c r="P9" s="19" t="n">
+        <v>0.09206273881812545</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>+37%</t>
-        </is>
-      </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>-171%</t>
-        </is>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>-2102bps</t>
-        </is>
-      </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>+68%</t>
-        </is>
-      </c>
-      <c r="F10" s="25" t="inlineStr">
-        <is>
-          <t>-203%</t>
-        </is>
-      </c>
-      <c r="G10" s="26" t="inlineStr">
-        <is>
-          <t>-2693bps</t>
-        </is>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>+65%</t>
-        </is>
-      </c>
-      <c r="I10" s="25" t="inlineStr">
-        <is>
-          <t>-180%</t>
-        </is>
-      </c>
-      <c r="J10" s="26" t="inlineStr">
-        <is>
-          <t>-1708bps</t>
-        </is>
-      </c>
-      <c r="K10" s="22" t="inlineStr">
-        <is>
-          <t>+93%</t>
-        </is>
-      </c>
-      <c r="L10" s="25" t="inlineStr">
-        <is>
-          <t>-232%</t>
-        </is>
-      </c>
-      <c r="M10" s="26" t="inlineStr">
-        <is>
-          <t>-2124bps</t>
-        </is>
-      </c>
-      <c r="N10" s="22" t="inlineStr">
-        <is>
-          <t>+50%</t>
-        </is>
-      </c>
-      <c r="O10" s="25" t="inlineStr">
-        <is>
-          <t>-189%</t>
-        </is>
-      </c>
-      <c r="P10" s="26" t="inlineStr">
-        <is>
-          <t>-2216bps</t>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>+35%</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>+1%</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>-267bps</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>+42%</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>-3%</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>-576bps</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>+30%</t>
+        </is>
+      </c>
+      <c r="I10" s="24" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>-649bps</t>
+        </is>
+      </c>
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>+71%</t>
+        </is>
+      </c>
+      <c r="L10" s="24" t="inlineStr">
+        <is>
+          <t>-39%</t>
+        </is>
+      </c>
+      <c r="M10" s="23" t="inlineStr">
+        <is>
+          <t>-867bps</t>
+        </is>
+      </c>
+      <c r="N10" s="21" t="inlineStr">
+        <is>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="O10" s="24" t="inlineStr">
+        <is>
+          <t>-8%</t>
+        </is>
+      </c>
+      <c r="P10" s="23" t="inlineStr">
+        <is>
+          <t>-469bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>6/7/2026</t>
+          <t>6/14/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>152258054</v>
+        <v>195613214</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>9252699</v>
+        <v>-14033670</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.06076984932435824</v>
+        <v>-0.07174193252609203</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>154759208</v>
+        <v>220845889</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>11517920</v>
+        <v>-22574161</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.07442477994588859</v>
+        <v>-0.1022168042258645</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>32812176</v>
+        <v>44703354</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>3627799</v>
+        <v>-2481951</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.1105625850598875</v>
+        <v>-0.05552046497450728</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>56847548</v>
+        <v>67325791</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>4335793</v>
+        <v>-5819762</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.07627053676967738</v>
+        <v>-0.08644179167534771</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>448604308</v>
+        <v>587580124</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>34132530</v>
+        <v>-48515978</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.07608605042642613</v>
+        <v>-0.08256912720213117</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t>+4%</t>
-        </is>
-      </c>
-      <c r="C12" s="29" t="inlineStr">
-        <is>
-          <t>-51%</t>
-        </is>
-      </c>
-      <c r="D12" s="30" t="inlineStr">
-        <is>
-          <t>-690bps</t>
-        </is>
-      </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t>+12%</t>
-        </is>
-      </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>-42%</t>
-        </is>
-      </c>
-      <c r="G12" s="30" t="inlineStr">
-        <is>
-          <t>-691bps</t>
-        </is>
-      </c>
-      <c r="H12" s="28" t="inlineStr">
-        <is>
-          <t>+15%</t>
-        </is>
-      </c>
-      <c r="I12" s="31" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>+37%</t>
         </is>
       </c>
-      <c r="J12" s="32" t="inlineStr">
-        <is>
-          <t>+179bps</t>
-        </is>
-      </c>
-      <c r="K12" s="28" t="inlineStr">
-        <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="L12" s="29" t="inlineStr">
-        <is>
-          <t>-1%</t>
-        </is>
-      </c>
-      <c r="M12" s="30" t="inlineStr">
-        <is>
-          <t>-430bps</t>
-        </is>
-      </c>
-      <c r="N12" s="28" t="inlineStr">
-        <is>
-          <t>+12%</t>
-        </is>
-      </c>
-      <c r="O12" s="29" t="inlineStr">
-        <is>
-          <t>-33%</t>
-        </is>
-      </c>
-      <c r="P12" s="30" t="inlineStr">
-        <is>
-          <t>-518bps</t>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>-171%</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>-2102bps</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>+68%</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>-203%</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>-2693bps</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>+65%</t>
+        </is>
+      </c>
+      <c r="I12" s="27" t="inlineStr">
+        <is>
+          <t>-180%</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="inlineStr">
+        <is>
+          <t>-1708bps</t>
+        </is>
+      </c>
+      <c r="K12" s="26" t="inlineStr">
+        <is>
+          <t>+93%</t>
+        </is>
+      </c>
+      <c r="L12" s="27" t="inlineStr">
+        <is>
+          <t>-232%</t>
+        </is>
+      </c>
+      <c r="M12" s="28" t="inlineStr">
+        <is>
+          <t>-2124bps</t>
+        </is>
+      </c>
+      <c r="N12" s="26" t="inlineStr">
+        <is>
+          <t>+50%</t>
+        </is>
+      </c>
+      <c r="O12" s="27" t="inlineStr">
+        <is>
+          <t>-189%</t>
+        </is>
+      </c>
+      <c r="P12" s="28" t="inlineStr">
+        <is>
+          <t>-2216bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Jul 23 19:00:54 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -216,6 +216,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -237,10 +240,10 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -249,10 +252,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -759,53 +765,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>7/12/2026</t>
+          <t>7/19/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>165737601</v>
+        <v>139807492</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>23467231</v>
+        <v>23125849</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.1415926793823931</v>
+        <v>0.1654120867857354</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>162520980</v>
+        <v>133999845</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>24960939</v>
+        <v>26554139</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.1535859493340491</v>
+        <v>0.1981654456391349</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>34868855</v>
+        <v>29900329</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>4459574</v>
+        <v>4363449</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.1278956249065248</v>
+        <v>0.1459331434112314</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>51411108</v>
+        <v>48553128</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>7470125</v>
+        <v>4987561</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.1453017701933209</v>
+        <v>0.1027237833162881</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>464461727</v>
+        <v>396178246</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>65981611</v>
+        <v>63579445</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.1420603833736337</v>
+        <v>0.1604819185352242</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -816,264 +822,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+35%</t>
+          <t>+39%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>+87%</t>
+          <t>+168%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>+391bps</t>
+          <t>+796bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+45%</t>
+          <t>+50%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>+65%</t>
+          <t>+83%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>+189bps</t>
+          <t>+358bps</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>+55%</t>
+          <t>+78%</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>+161%</t>
+          <t>+96%</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>+520bps</t>
+          <t>+137bps</t>
         </is>
       </c>
       <c r="K4" s="13" t="inlineStr">
         <is>
-          <t>+68%</t>
+          <t>+72%</t>
         </is>
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>+519bps</t>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
+          <t>-96bps</t>
         </is>
       </c>
       <c r="N4" s="13" t="inlineStr">
         <is>
-          <t>+41%</t>
+          <t>+49%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>+89%</t>
+          <t>+98%</t>
         </is>
       </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
-          <t>+356bps</t>
+          <t>+399bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>7/5/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="n">
-        <v>198331851</v>
-      </c>
-      <c r="C5" s="18" t="n">
-        <v>13762042</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>0.06938896566845433</v>
-      </c>
-      <c r="E5" s="17" t="n">
-        <v>187715921</v>
-      </c>
-      <c r="F5" s="18" t="n">
-        <v>13578971</v>
-      </c>
-      <c r="G5" s="19" t="n">
-        <v>0.07233787591197445</v>
-      </c>
-      <c r="H5" s="17" t="n">
-        <v>39155250</v>
-      </c>
-      <c r="I5" s="18" t="n">
-        <v>2644188</v>
-      </c>
-      <c r="J5" s="19" t="n">
-        <v>0.06753086750818856</v>
-      </c>
-      <c r="K5" s="17" t="n">
-        <v>62287631</v>
-      </c>
-      <c r="L5" s="18" t="n">
-        <v>3223781</v>
-      </c>
-      <c r="M5" s="19" t="n">
-        <v>0.05175635913974638</v>
-      </c>
-      <c r="N5" s="17" t="n">
-        <v>548797512</v>
-      </c>
-      <c r="O5" s="18" t="n">
-        <v>36510807</v>
-      </c>
-      <c r="P5" s="19" t="n">
-        <v>0.06652874002096423</v>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>7/12/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>165737601</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>23467231</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>0.1415926793823931</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>162520980</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>24960939</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>0.1535859493340491</v>
+      </c>
+      <c r="H5" s="18" t="n">
+        <v>34868855</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>4459574</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <v>0.1278956249065248</v>
+      </c>
+      <c r="K5" s="18" t="n">
+        <v>51411108</v>
+      </c>
+      <c r="L5" s="19" t="n">
+        <v>7470125</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>0.1453017701933209</v>
+      </c>
+      <c r="N5" s="18" t="n">
+        <v>464461727</v>
+      </c>
+      <c r="O5" s="19" t="n">
+        <v>65981611</v>
+      </c>
+      <c r="P5" s="20" t="n">
+        <v>0.1420603833736337</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>+48%</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="inlineStr">
-        <is>
-          <t>+2%</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>-319bps</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>+57%</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>+1%</t>
-        </is>
-      </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>-407bps</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>+60%</t>
-        </is>
-      </c>
-      <c r="I6" s="22" t="inlineStr">
-        <is>
-          <t>+20%</t>
-        </is>
-      </c>
-      <c r="J6" s="23" t="inlineStr">
-        <is>
-          <t>-223bps</t>
-        </is>
-      </c>
-      <c r="K6" s="21" t="inlineStr">
-        <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="L6" s="24" t="inlineStr">
-        <is>
-          <t>-9%</t>
-        </is>
-      </c>
-      <c r="M6" s="23" t="inlineStr">
-        <is>
-          <t>-612bps</t>
-        </is>
-      </c>
-      <c r="N6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>+35%</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>+87%</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>+391bps</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>+45%</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>+65%</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>+189bps</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>+55%</t>
         </is>
       </c>
-      <c r="O6" s="24" t="inlineStr">
-        <is>
-          <t>-4%</t>
-        </is>
-      </c>
-      <c r="P6" s="23" t="inlineStr">
-        <is>
-          <t>-410bps</t>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>+161%</t>
+        </is>
+      </c>
+      <c r="J6" s="24" t="inlineStr">
+        <is>
+          <t>+520bps</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="inlineStr">
+        <is>
+          <t>+68%</t>
+        </is>
+      </c>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>+161%</t>
+        </is>
+      </c>
+      <c r="M6" s="24" t="inlineStr">
+        <is>
+          <t>+519bps</t>
+        </is>
+      </c>
+      <c r="N6" s="22" t="inlineStr">
+        <is>
+          <t>+41%</t>
+        </is>
+      </c>
+      <c r="O6" s="23" t="inlineStr">
+        <is>
+          <t>+89%</t>
+        </is>
+      </c>
+      <c r="P6" s="24" t="inlineStr">
+        <is>
+          <t>+356bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>6/28/2026</t>
+          <t>7/5/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>187265340</v>
+        <v>198331851</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>20773685</v>
+        <v>13762042</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.1109318200581058</v>
+        <v>0.06938896566845433</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>178427790</v>
+        <v>187715921</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>25667736</v>
+        <v>13578971</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1438550351377439</v>
+        <v>0.07233787591197445</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>34322403</v>
+        <v>39155250</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>4555167</v>
+        <v>2644188</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.1327170186772762</v>
+        <v>0.06753086750818856</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>59305990</v>
+        <v>62287631</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>5238538</v>
+        <v>3223781</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.08833067283760039</v>
+        <v>0.05175635913974638</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>512508333</v>
+        <v>548797512</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>61849542</v>
+        <v>36510807</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.120680070971646</v>
+        <v>0.06652874002096423</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1084,345 +1090,345 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>+45%</t>
+          <t>+48%</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>+306bps</t>
+          <t>+2%</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>-319bps</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>+49%</t>
+          <t>+57%</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>+67%</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>+158bps</t>
+          <t>+1%</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>-407bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+38%</t>
+          <t>+60%</t>
         </is>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
-          <t>+417%</t>
-        </is>
-      </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>+974bps</t>
+          <t>+20%</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>-223bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>+73%</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>+117bps</t>
+          <t>+98%</t>
+        </is>
+      </c>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>-9%</t>
+        </is>
+      </c>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>-612bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="O8" s="14" t="inlineStr">
-        <is>
-          <t>+86%</t>
-        </is>
-      </c>
-      <c r="P8" s="15" t="inlineStr">
-        <is>
-          <t>+255bps</t>
+          <t>+55%</t>
+        </is>
+      </c>
+      <c r="O8" s="25" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="P8" s="16" t="inlineStr">
+        <is>
+          <t>-410bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>6/21/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="n">
-        <v>196191527</v>
-      </c>
-      <c r="C9" s="18" t="n">
-        <v>15707056</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>0.08005980808743081</v>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>197643614</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>24458285</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>0.1237494321470968</v>
-      </c>
-      <c r="H9" s="17" t="n">
-        <v>37762064</v>
-      </c>
-      <c r="I9" s="18" t="n">
-        <v>3330257</v>
-      </c>
-      <c r="J9" s="19" t="n">
-        <v>0.08819054488123319</v>
-      </c>
-      <c r="K9" s="17" t="n">
-        <v>64128131</v>
-      </c>
-      <c r="L9" s="18" t="n">
-        <v>3055347</v>
-      </c>
-      <c r="M9" s="19" t="n">
-        <v>0.04764441053178362</v>
-      </c>
-      <c r="N9" s="17" t="n">
-        <v>551320172</v>
-      </c>
-      <c r="O9" s="18" t="n">
-        <v>50756045</v>
-      </c>
-      <c r="P9" s="19" t="n">
-        <v>0.09206273881812545</v>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>6/28/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>187265340</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>20773685</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>0.1109318200581058</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>178427790</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>25667736</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>0.1438550351377439</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>34322403</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>4555167</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>0.1327170186772762</v>
+      </c>
+      <c r="K9" s="18" t="n">
+        <v>59305990</v>
+      </c>
+      <c r="L9" s="19" t="n">
+        <v>5238538</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <v>0.08833067283760039</v>
+      </c>
+      <c r="N9" s="18" t="n">
+        <v>512508333</v>
+      </c>
+      <c r="O9" s="19" t="n">
+        <v>61849542</v>
+      </c>
+      <c r="P9" s="20" t="n">
+        <v>0.120680070971646</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>+35%</t>
-        </is>
-      </c>
-      <c r="C10" s="22" t="inlineStr">
-        <is>
-          <t>+1%</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>-267bps</t>
-        </is>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
-          <t>+42%</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr">
-        <is>
-          <t>-3%</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>-576bps</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="inlineStr">
-        <is>
-          <t>+30%</t>
-        </is>
-      </c>
-      <c r="I10" s="24" t="inlineStr">
-        <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="J10" s="23" t="inlineStr">
-        <is>
-          <t>-649bps</t>
-        </is>
-      </c>
-      <c r="K10" s="21" t="inlineStr">
-        <is>
-          <t>+71%</t>
-        </is>
-      </c>
-      <c r="L10" s="24" t="inlineStr">
-        <is>
-          <t>-39%</t>
-        </is>
-      </c>
-      <c r="M10" s="23" t="inlineStr">
-        <is>
-          <t>-867bps</t>
-        </is>
-      </c>
-      <c r="N10" s="21" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>+45%</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>+100%</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>+306bps</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>+49%</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>+67%</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>+158bps</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>+38%</t>
         </is>
       </c>
-      <c r="O10" s="24" t="inlineStr">
-        <is>
-          <t>-8%</t>
-        </is>
-      </c>
-      <c r="P10" s="23" t="inlineStr">
-        <is>
-          <t>-469bps</t>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>+417%</t>
+        </is>
+      </c>
+      <c r="J10" s="24" t="inlineStr">
+        <is>
+          <t>+974bps</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="inlineStr">
+        <is>
+          <t>+73%</t>
+        </is>
+      </c>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>+100%</t>
+        </is>
+      </c>
+      <c r="M10" s="24" t="inlineStr">
+        <is>
+          <t>+117bps</t>
+        </is>
+      </c>
+      <c r="N10" s="22" t="inlineStr">
+        <is>
+          <t>+47%</t>
+        </is>
+      </c>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>+86%</t>
+        </is>
+      </c>
+      <c r="P10" s="24" t="inlineStr">
+        <is>
+          <t>+255bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>6/14/2026</t>
+          <t>6/21/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>195613214</v>
+        <v>196191527</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>-14033670</v>
+        <v>15707056</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>-0.07174193252609203</v>
+        <v>0.08005980808743081</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>220845889</v>
+        <v>197643614</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>-22574161</v>
+        <v>24458285</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>-0.1022168042258645</v>
+        <v>0.1237494321470968</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>44703354</v>
+        <v>37762064</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>-2481951</v>
+        <v>3330257</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>-0.05552046497450728</v>
+        <v>0.08819054488123319</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>67325791</v>
+        <v>64128131</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>-5819762</v>
+        <v>3055347</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>-0.08644179167534771</v>
+        <v>0.04764441053178362</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>587580124</v>
+        <v>551320172</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>-48515978</v>
+        <v>50756045</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>-0.08256912720213117</v>
+        <v>0.09206273881812545</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>+37%</t>
-        </is>
-      </c>
-      <c r="C12" s="27" t="inlineStr">
-        <is>
-          <t>-171%</t>
-        </is>
-      </c>
-      <c r="D12" s="28" t="inlineStr">
-        <is>
-          <t>-2102bps</t>
-        </is>
-      </c>
-      <c r="E12" s="26" t="inlineStr">
-        <is>
-          <t>+68%</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="inlineStr">
-        <is>
-          <t>-203%</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="inlineStr">
-        <is>
-          <t>-2693bps</t>
-        </is>
-      </c>
-      <c r="H12" s="26" t="inlineStr">
-        <is>
-          <t>+65%</t>
-        </is>
-      </c>
-      <c r="I12" s="27" t="inlineStr">
-        <is>
-          <t>-180%</t>
-        </is>
-      </c>
-      <c r="J12" s="28" t="inlineStr">
-        <is>
-          <t>-1708bps</t>
-        </is>
-      </c>
-      <c r="K12" s="26" t="inlineStr">
-        <is>
-          <t>+93%</t>
-        </is>
-      </c>
-      <c r="L12" s="27" t="inlineStr">
-        <is>
-          <t>-232%</t>
-        </is>
-      </c>
-      <c r="M12" s="28" t="inlineStr">
-        <is>
-          <t>-2124bps</t>
-        </is>
-      </c>
-      <c r="N12" s="26" t="inlineStr">
-        <is>
-          <t>+50%</t>
-        </is>
-      </c>
-      <c r="O12" s="27" t="inlineStr">
-        <is>
-          <t>-189%</t>
-        </is>
-      </c>
-      <c r="P12" s="28" t="inlineStr">
-        <is>
-          <t>-2216bps</t>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>+35%</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>+1%</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>-267bps</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>+42%</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>-3%</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>-576bps</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="inlineStr">
+        <is>
+          <t>+30%</t>
+        </is>
+      </c>
+      <c r="I12" s="30" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>-649bps</t>
+        </is>
+      </c>
+      <c r="K12" s="27" t="inlineStr">
+        <is>
+          <t>+71%</t>
+        </is>
+      </c>
+      <c r="L12" s="30" t="inlineStr">
+        <is>
+          <t>-39%</t>
+        </is>
+      </c>
+      <c r="M12" s="29" t="inlineStr">
+        <is>
+          <t>-867bps</t>
+        </is>
+      </c>
+      <c r="N12" s="27" t="inlineStr">
+        <is>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="O12" s="30" t="inlineStr">
+        <is>
+          <t>-8%</t>
+        </is>
+      </c>
+      <c r="P12" s="29" t="inlineStr">
+        <is>
+          <t>-469bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Fri Jul 31 15:30:53 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,15 +210,18 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -243,7 +246,10 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -255,10 +261,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -765,53 +768,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>7/19/2026</t>
+          <t>7/26/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>139807492</v>
+        <v>121558881</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>23125849</v>
+        <v>8980474</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.1654120867857354</v>
+        <v>0.0738775639107767</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>133999845</v>
+        <v>123109037</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>26554139</v>
+        <v>10499562</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.1981654456391349</v>
+        <v>0.08528668776769004</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>29900329</v>
+        <v>24313828</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>4363449</v>
+        <v>2831499</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.1459331434112314</v>
+        <v>0.1164563227147942</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>48553128</v>
+        <v>45125668</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>4987561</v>
+        <v>2828135</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.1027237833162881</v>
+        <v>0.06267242404034883</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>396178246</v>
+        <v>354055496</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>63579445</v>
+        <v>27911568</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.1604819185352242</v>
+        <v>0.0788338786301456</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -822,264 +825,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+39%</t>
+          <t>+6%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>+168%</t>
+          <t>-28%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>+796bps</t>
+          <t>-347bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+50%</t>
+          <t>+8%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>+83%</t>
+          <t>-11%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>+358bps</t>
+          <t>-186bps</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>+78%</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>+96%</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>+137bps</t>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>+13%</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>+76bps</t>
         </is>
       </c>
       <c r="K4" s="13" t="inlineStr">
         <is>
-          <t>+72%</t>
+          <t>+44%</t>
         </is>
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>+57%</t>
-        </is>
-      </c>
-      <c r="M4" s="16" t="inlineStr">
-        <is>
-          <t>-96bps</t>
+          <t>-24%</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>-554bps</t>
         </is>
       </c>
       <c r="N4" s="13" t="inlineStr">
         <is>
-          <t>+49%</t>
+          <t>+8%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>+98%</t>
+          <t>-20%</t>
         </is>
       </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
-          <t>+399bps</t>
+          <t>-273bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>7/12/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="n">
-        <v>165737601</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>23467231</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.1415926793823931</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>162520980</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>24960939</v>
-      </c>
-      <c r="G5" s="20" t="n">
-        <v>0.1535859493340491</v>
-      </c>
-      <c r="H5" s="18" t="n">
-        <v>34868855</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>4459574</v>
-      </c>
-      <c r="J5" s="20" t="n">
-        <v>0.1278956249065248</v>
-      </c>
-      <c r="K5" s="18" t="n">
-        <v>51411108</v>
-      </c>
-      <c r="L5" s="19" t="n">
-        <v>7470125</v>
-      </c>
-      <c r="M5" s="20" t="n">
-        <v>0.1453017701933209</v>
-      </c>
-      <c r="N5" s="18" t="n">
-        <v>464461727</v>
-      </c>
-      <c r="O5" s="19" t="n">
-        <v>65981611</v>
-      </c>
-      <c r="P5" s="20" t="n">
-        <v>0.1420603833736337</v>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>7/19/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>139807492</v>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>23125849</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>0.1654120867857354</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>133999845</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>26554139</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>0.1981654456391349</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>29900329</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>4363449</v>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>0.1459331434112314</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>48553128</v>
+      </c>
+      <c r="L5" s="20" t="n">
+        <v>4987561</v>
+      </c>
+      <c r="M5" s="21" t="n">
+        <v>0.1027237833162881</v>
+      </c>
+      <c r="N5" s="19" t="n">
+        <v>396178246</v>
+      </c>
+      <c r="O5" s="20" t="n">
+        <v>63579445</v>
+      </c>
+      <c r="P5" s="21" t="n">
+        <v>0.1604819185352242</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>+35%</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>+87%</t>
-        </is>
-      </c>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>+391bps</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>+65%</t>
-        </is>
-      </c>
-      <c r="G6" s="24" t="inlineStr">
-        <is>
-          <t>+189bps</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="I6" s="23" t="inlineStr">
-        <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="J6" s="24" t="inlineStr">
-        <is>
-          <t>+520bps</t>
-        </is>
-      </c>
-      <c r="K6" s="22" t="inlineStr">
-        <is>
-          <t>+68%</t>
-        </is>
-      </c>
-      <c r="L6" s="23" t="inlineStr">
-        <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="M6" s="24" t="inlineStr">
-        <is>
-          <t>+519bps</t>
-        </is>
-      </c>
-      <c r="N6" s="22" t="inlineStr">
-        <is>
-          <t>+41%</t>
-        </is>
-      </c>
-      <c r="O6" s="23" t="inlineStr">
-        <is>
-          <t>+89%</t>
-        </is>
-      </c>
-      <c r="P6" s="24" t="inlineStr">
-        <is>
-          <t>+356bps</t>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>+39%</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>+168%</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>+796bps</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>+50%</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>+83%</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>+358bps</t>
+        </is>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>+78%</t>
+        </is>
+      </c>
+      <c r="I6" s="24" t="inlineStr">
+        <is>
+          <t>+96%</t>
+        </is>
+      </c>
+      <c r="J6" s="25" t="inlineStr">
+        <is>
+          <t>+137bps</t>
+        </is>
+      </c>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>+72%</t>
+        </is>
+      </c>
+      <c r="L6" s="24" t="inlineStr">
+        <is>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="M6" s="26" t="inlineStr">
+        <is>
+          <t>-96bps</t>
+        </is>
+      </c>
+      <c r="N6" s="23" t="inlineStr">
+        <is>
+          <t>+49%</t>
+        </is>
+      </c>
+      <c r="O6" s="24" t="inlineStr">
+        <is>
+          <t>+98%</t>
+        </is>
+      </c>
+      <c r="P6" s="25" t="inlineStr">
+        <is>
+          <t>+399bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>7/5/2026</t>
+          <t>7/12/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>198331851</v>
+        <v>165737601</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>13762042</v>
+        <v>23467231</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.06938896566845433</v>
+        <v>0.1415926793823931</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>187715921</v>
+        <v>162520980</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>13578971</v>
+        <v>24960939</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.07233787591197445</v>
+        <v>0.1535859493340491</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>39155250</v>
+        <v>34868855</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>2644188</v>
+        <v>4459574</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.06753086750818856</v>
+        <v>0.1278956249065248</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>62287631</v>
+        <v>51411108</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>3223781</v>
+        <v>7470125</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.05175635913974638</v>
+        <v>0.1453017701933209</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>548797512</v>
+        <v>464461727</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>36510807</v>
+        <v>65981611</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.06652874002096423</v>
+        <v>0.1420603833736337</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1090,345 +1093,345 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>+48%</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>+2%</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>-319bps</t>
+          <t>+35%</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>+87%</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>+391bps</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>+57%</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>+1%</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>-407bps</t>
+          <t>+45%</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>+65%</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>+189bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+60%</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>+20%</t>
-        </is>
-      </c>
-      <c r="J8" s="16" t="inlineStr">
-        <is>
-          <t>-223bps</t>
+          <t>+55%</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>+161%</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t>+520bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="L8" s="25" t="inlineStr">
-        <is>
-          <t>-9%</t>
-        </is>
-      </c>
-      <c r="M8" s="16" t="inlineStr">
-        <is>
-          <t>-612bps</t>
+          <t>+68%</t>
+        </is>
+      </c>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>+161%</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>+519bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="O8" s="25" t="inlineStr">
-        <is>
-          <t>-4%</t>
-        </is>
-      </c>
-      <c r="P8" s="16" t="inlineStr">
-        <is>
-          <t>-410bps</t>
+          <t>+41%</t>
+        </is>
+      </c>
+      <c r="O8" s="16" t="inlineStr">
+        <is>
+          <t>+89%</t>
+        </is>
+      </c>
+      <c r="P8" s="17" t="inlineStr">
+        <is>
+          <t>+356bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>6/28/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>187265340</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>20773685</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0.1109318200581058</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>178427790</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>25667736</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>0.1438550351377439</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>34322403</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>4555167</v>
-      </c>
-      <c r="J9" s="20" t="n">
-        <v>0.1327170186772762</v>
-      </c>
-      <c r="K9" s="18" t="n">
-        <v>59305990</v>
-      </c>
-      <c r="L9" s="19" t="n">
-        <v>5238538</v>
-      </c>
-      <c r="M9" s="20" t="n">
-        <v>0.08833067283760039</v>
-      </c>
-      <c r="N9" s="18" t="n">
-        <v>512508333</v>
-      </c>
-      <c r="O9" s="19" t="n">
-        <v>61849542</v>
-      </c>
-      <c r="P9" s="20" t="n">
-        <v>0.120680070971646</v>
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>7/5/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>198331851</v>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>13762042</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0.06938896566845433</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>187715921</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>13578971</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>0.07233787591197445</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>39155250</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>2644188</v>
+      </c>
+      <c r="J9" s="21" t="n">
+        <v>0.06753086750818856</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>62287631</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>3223781</v>
+      </c>
+      <c r="M9" s="21" t="n">
+        <v>0.05175635913974638</v>
+      </c>
+      <c r="N9" s="19" t="n">
+        <v>548797512</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <v>36510807</v>
+      </c>
+      <c r="P9" s="21" t="n">
+        <v>0.06652874002096423</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>+306bps</t>
-        </is>
-      </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>+49%</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>+67%</t>
-        </is>
-      </c>
-      <c r="G10" s="24" t="inlineStr">
-        <is>
-          <t>+158bps</t>
-        </is>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="I10" s="23" t="inlineStr">
-        <is>
-          <t>+417%</t>
-        </is>
-      </c>
-      <c r="J10" s="24" t="inlineStr">
-        <is>
-          <t>+974bps</t>
-        </is>
-      </c>
-      <c r="K10" s="22" t="inlineStr">
-        <is>
-          <t>+73%</t>
-        </is>
-      </c>
-      <c r="L10" s="23" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="M10" s="24" t="inlineStr">
-        <is>
-          <t>+117bps</t>
-        </is>
-      </c>
-      <c r="N10" s="22" t="inlineStr">
-        <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="O10" s="23" t="inlineStr">
-        <is>
-          <t>+86%</t>
-        </is>
-      </c>
-      <c r="P10" s="24" t="inlineStr">
-        <is>
-          <t>+255bps</t>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>+2%</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>-319bps</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>+1%</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>-407bps</t>
+        </is>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>+60%</t>
+        </is>
+      </c>
+      <c r="I10" s="24" t="inlineStr">
+        <is>
+          <t>+20%</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t>-223bps</t>
+        </is>
+      </c>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>+98%</t>
+        </is>
+      </c>
+      <c r="L10" s="27" t="inlineStr">
+        <is>
+          <t>-9%</t>
+        </is>
+      </c>
+      <c r="M10" s="26" t="inlineStr">
+        <is>
+          <t>-612bps</t>
+        </is>
+      </c>
+      <c r="N10" s="23" t="inlineStr">
+        <is>
+          <t>+55%</t>
+        </is>
+      </c>
+      <c r="O10" s="27" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="P10" s="26" t="inlineStr">
+        <is>
+          <t>-410bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>6/21/2026</t>
+          <t>6/28/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>196191527</v>
+        <v>187265340</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>15707056</v>
+        <v>20773685</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.08005980808743081</v>
+        <v>0.1109318200581058</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>197643614</v>
+        <v>178427790</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>24458285</v>
+        <v>25667736</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.1237494321470968</v>
+        <v>0.1438550351377439</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>37762064</v>
+        <v>34322403</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>3330257</v>
+        <v>4555167</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.08819054488123319</v>
+        <v>0.1327170186772762</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>64128131</v>
+        <v>59305990</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>3055347</v>
+        <v>5238538</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.04764441053178362</v>
+        <v>0.08833067283760039</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>551320172</v>
+        <v>512508333</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>50756045</v>
+        <v>61849542</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.09206273881812545</v>
+        <v>0.120680070971646</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>+35%</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="inlineStr">
-        <is>
-          <t>+1%</t>
-        </is>
-      </c>
-      <c r="D12" s="29" t="inlineStr">
-        <is>
-          <t>-267bps</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="inlineStr">
-        <is>
-          <t>+42%</t>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>+45%</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>+100%</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>+306bps</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="inlineStr">
+        <is>
+          <t>+49%</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>-3%</t>
-        </is>
-      </c>
-      <c r="G12" s="29" t="inlineStr">
-        <is>
-          <t>-576bps</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="inlineStr">
-        <is>
-          <t>+30%</t>
+          <t>+67%</t>
+        </is>
+      </c>
+      <c r="G12" s="31" t="inlineStr">
+        <is>
+          <t>+158bps</t>
+        </is>
+      </c>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>+38%</t>
         </is>
       </c>
       <c r="I12" s="30" t="inlineStr">
         <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="J12" s="29" t="inlineStr">
-        <is>
-          <t>-649bps</t>
-        </is>
-      </c>
-      <c r="K12" s="27" t="inlineStr">
-        <is>
-          <t>+71%</t>
+          <t>+417%</t>
+        </is>
+      </c>
+      <c r="J12" s="31" t="inlineStr">
+        <is>
+          <t>+974bps</t>
+        </is>
+      </c>
+      <c r="K12" s="29" t="inlineStr">
+        <is>
+          <t>+73%</t>
         </is>
       </c>
       <c r="L12" s="30" t="inlineStr">
         <is>
-          <t>-39%</t>
-        </is>
-      </c>
-      <c r="M12" s="29" t="inlineStr">
-        <is>
-          <t>-867bps</t>
-        </is>
-      </c>
-      <c r="N12" s="27" t="inlineStr">
-        <is>
-          <t>+38%</t>
+          <t>+100%</t>
+        </is>
+      </c>
+      <c r="M12" s="31" t="inlineStr">
+        <is>
+          <t>+117bps</t>
+        </is>
+      </c>
+      <c r="N12" s="29" t="inlineStr">
+        <is>
+          <t>+47%</t>
         </is>
       </c>
       <c r="O12" s="30" t="inlineStr">
         <is>
-          <t>-8%</t>
-        </is>
-      </c>
-      <c r="P12" s="29" t="inlineStr">
-        <is>
-          <t>-469bps</t>
+          <t>+86%</t>
+        </is>
+      </c>
+      <c r="P12" s="31" t="inlineStr">
+        <is>
+          <t>+255bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Aug  6 20:00:58 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,13 +210,16 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,18 +243,18 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -261,7 +264,10 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -768,53 +774,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>7/26/2026</t>
+          <t>8/2/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>121558881</v>
+        <v>130246036</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>8980474</v>
+        <v>16204920</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.0738775639107767</v>
+        <v>0.1244177596314716</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>123109037</v>
+        <v>136855999</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>10499562</v>
+        <v>18214019</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.08528668776769004</v>
+        <v>0.133088933865442</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>24313828</v>
+        <v>33134991</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>2831499</v>
+        <v>2695236</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.1164563227147942</v>
+        <v>0.08134108139640056</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>45125668</v>
+        <v>43379501</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>2828135</v>
+        <v>5473675</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.06267242404034883</v>
+        <v>0.126181142563166</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>354055496</v>
+        <v>384761041</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>27911568</v>
+        <v>46532432</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.0788338786301456</v>
+        <v>0.120938522983152</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -825,264 +831,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+6%</t>
+          <t>+18%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>-28%</t>
+          <t>+13%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>-347bps</t>
+          <t>-58bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+8%</t>
+          <t>+22%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>-11%</t>
+          <t>+9%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>-186bps</t>
+          <t>-163bps</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>+5%</t>
+          <t>+23%</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="J4" s="17" t="inlineStr">
-        <is>
-          <t>+76bps</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>+44%</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>-24%</t>
-        </is>
-      </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>-554bps</t>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>-559bps</t>
+        </is>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
+          <t>-7%</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
+          <t>-243%</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>+2082bps</t>
         </is>
       </c>
       <c r="N4" s="13" t="inlineStr">
         <is>
-          <t>+8%</t>
+          <t>+14%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>-20%</t>
-        </is>
-      </c>
-      <c r="P4" s="15" t="inlineStr">
-        <is>
-          <t>-273bps</t>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="P4" s="18" t="inlineStr">
+        <is>
+          <t>+140bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>7/19/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>139807492</v>
-      </c>
-      <c r="C5" s="20" t="n">
-        <v>23125849</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>0.1654120867857354</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>133999845</v>
-      </c>
-      <c r="F5" s="20" t="n">
-        <v>26554139</v>
-      </c>
-      <c r="G5" s="21" t="n">
-        <v>0.1981654456391349</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>29900329</v>
-      </c>
-      <c r="I5" s="20" t="n">
-        <v>4363449</v>
-      </c>
-      <c r="J5" s="21" t="n">
-        <v>0.1459331434112314</v>
-      </c>
-      <c r="K5" s="19" t="n">
-        <v>48553128</v>
-      </c>
-      <c r="L5" s="20" t="n">
-        <v>4987561</v>
-      </c>
-      <c r="M5" s="21" t="n">
-        <v>0.1027237833162881</v>
-      </c>
-      <c r="N5" s="19" t="n">
-        <v>396178246</v>
-      </c>
-      <c r="O5" s="20" t="n">
-        <v>63579445</v>
-      </c>
-      <c r="P5" s="21" t="n">
-        <v>0.1604819185352242</v>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>7/26/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>121558881</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>8980474</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>0.0738775639107767</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>123109037</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>10499562</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.08528668776769004</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>24313828</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>2831499</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.1164563227147942</v>
+      </c>
+      <c r="K5" s="20" t="n">
+        <v>45125668</v>
+      </c>
+      <c r="L5" s="21" t="n">
+        <v>2828135</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.06267242404034883</v>
+      </c>
+      <c r="N5" s="20" t="n">
+        <v>354055496</v>
+      </c>
+      <c r="O5" s="21" t="n">
+        <v>27911568</v>
+      </c>
+      <c r="P5" s="22" t="n">
+        <v>0.0788338786301456</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>+39%</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>+168%</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>+796bps</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>+50%</t>
-        </is>
-      </c>
-      <c r="F6" s="24" t="inlineStr">
-        <is>
-          <t>+83%</t>
-        </is>
-      </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>+358bps</t>
-        </is>
-      </c>
-      <c r="H6" s="23" t="inlineStr">
-        <is>
-          <t>+78%</t>
-        </is>
-      </c>
-      <c r="I6" s="24" t="inlineStr">
-        <is>
-          <t>+96%</t>
-        </is>
-      </c>
-      <c r="J6" s="25" t="inlineStr">
-        <is>
-          <t>+137bps</t>
-        </is>
-      </c>
-      <c r="K6" s="23" t="inlineStr">
-        <is>
-          <t>+72%</t>
-        </is>
-      </c>
-      <c r="L6" s="24" t="inlineStr">
-        <is>
-          <t>+57%</t>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>+6%</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>-28%</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>-347bps</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>-186bps</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>+13%</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>+76bps</t>
+        </is>
+      </c>
+      <c r="K6" s="24" t="inlineStr">
+        <is>
+          <t>+44%</t>
+        </is>
+      </c>
+      <c r="L6" s="25" t="inlineStr">
+        <is>
+          <t>-24%</t>
         </is>
       </c>
       <c r="M6" s="26" t="inlineStr">
         <is>
-          <t>-96bps</t>
-        </is>
-      </c>
-      <c r="N6" s="23" t="inlineStr">
-        <is>
-          <t>+49%</t>
-        </is>
-      </c>
-      <c r="O6" s="24" t="inlineStr">
-        <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="P6" s="25" t="inlineStr">
-        <is>
-          <t>+399bps</t>
+          <t>-554bps</t>
+        </is>
+      </c>
+      <c r="N6" s="24" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="O6" s="25" t="inlineStr">
+        <is>
+          <t>-20%</t>
+        </is>
+      </c>
+      <c r="P6" s="26" t="inlineStr">
+        <is>
+          <t>-273bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>7/12/2026</t>
+          <t>7/19/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>165737601</v>
+        <v>139807492</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>23467231</v>
+        <v>23125849</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.1415926793823931</v>
+        <v>0.1654120867857354</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>162520980</v>
+        <v>133999845</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>24960939</v>
+        <v>26554139</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1535859493340491</v>
+        <v>0.1981654456391349</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>34868855</v>
+        <v>29900329</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>4459574</v>
+        <v>4363449</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.1278956249065248</v>
+        <v>0.1459331434112314</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>51411108</v>
+        <v>48553128</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>7470125</v>
+        <v>4987561</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.1453017701933209</v>
+        <v>0.1027237833162881</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>464461727</v>
+        <v>396178246</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>65981611</v>
+        <v>63579445</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.1420603833736337</v>
+        <v>0.1604819185352242</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1093,345 +1099,345 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>+35%</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>+87%</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>+391bps</t>
+          <t>+39%</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>+168%</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>+796bps</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>+65%</t>
-        </is>
-      </c>
-      <c r="G8" s="17" t="inlineStr">
-        <is>
-          <t>+189bps</t>
+          <t>+50%</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>+83%</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>+358bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="J8" s="17" t="inlineStr">
-        <is>
-          <t>+520bps</t>
+          <t>+78%</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>+96%</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>+137bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>+68%</t>
-        </is>
-      </c>
-      <c r="L8" s="16" t="inlineStr">
-        <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="M8" s="17" t="inlineStr">
-        <is>
-          <t>+519bps</t>
+          <t>+72%</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>-96bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+41%</t>
-        </is>
-      </c>
-      <c r="O8" s="16" t="inlineStr">
-        <is>
-          <t>+89%</t>
-        </is>
-      </c>
-      <c r="P8" s="17" t="inlineStr">
-        <is>
-          <t>+356bps</t>
+          <t>+49%</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>+98%</t>
+        </is>
+      </c>
+      <c r="P8" s="18" t="inlineStr">
+        <is>
+          <t>+399bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>7/5/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>198331851</v>
-      </c>
-      <c r="C9" s="20" t="n">
-        <v>13762042</v>
-      </c>
-      <c r="D9" s="21" t="n">
-        <v>0.06938896566845433</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>187715921</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>13578971</v>
-      </c>
-      <c r="G9" s="21" t="n">
-        <v>0.07233787591197445</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>39155250</v>
-      </c>
-      <c r="I9" s="20" t="n">
-        <v>2644188</v>
-      </c>
-      <c r="J9" s="21" t="n">
-        <v>0.06753086750818856</v>
-      </c>
-      <c r="K9" s="19" t="n">
-        <v>62287631</v>
-      </c>
-      <c r="L9" s="20" t="n">
-        <v>3223781</v>
-      </c>
-      <c r="M9" s="21" t="n">
-        <v>0.05175635913974638</v>
-      </c>
-      <c r="N9" s="19" t="n">
-        <v>548797512</v>
-      </c>
-      <c r="O9" s="20" t="n">
-        <v>36510807</v>
-      </c>
-      <c r="P9" s="21" t="n">
-        <v>0.06652874002096423</v>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>7/12/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>165737601</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>23467231</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.1415926793823931</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>162520980</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>24960939</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>0.1535859493340491</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>34868855</v>
+      </c>
+      <c r="I9" s="21" t="n">
+        <v>4459574</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.1278956249065248</v>
+      </c>
+      <c r="K9" s="20" t="n">
+        <v>51411108</v>
+      </c>
+      <c r="L9" s="21" t="n">
+        <v>7470125</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>0.1453017701933209</v>
+      </c>
+      <c r="N9" s="20" t="n">
+        <v>464461727</v>
+      </c>
+      <c r="O9" s="21" t="n">
+        <v>65981611</v>
+      </c>
+      <c r="P9" s="22" t="n">
+        <v>0.1420603833736337</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>+48%</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>+2%</t>
-        </is>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>-319bps</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>+57%</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr">
-        <is>
-          <t>+1%</t>
-        </is>
-      </c>
-      <c r="G10" s="26" t="inlineStr">
-        <is>
-          <t>-407bps</t>
-        </is>
-      </c>
-      <c r="H10" s="23" t="inlineStr">
-        <is>
-          <t>+60%</t>
-        </is>
-      </c>
-      <c r="I10" s="24" t="inlineStr">
-        <is>
-          <t>+20%</t>
-        </is>
-      </c>
-      <c r="J10" s="26" t="inlineStr">
-        <is>
-          <t>-223bps</t>
-        </is>
-      </c>
-      <c r="K10" s="23" t="inlineStr">
-        <is>
-          <t>+98%</t>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>+35%</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>+87%</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>+391bps</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>+45%</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>+65%</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>+189bps</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>+55%</t>
+        </is>
+      </c>
+      <c r="I10" s="27" t="inlineStr">
+        <is>
+          <t>+161%</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="inlineStr">
+        <is>
+          <t>+520bps</t>
+        </is>
+      </c>
+      <c r="K10" s="24" t="inlineStr">
+        <is>
+          <t>+68%</t>
         </is>
       </c>
       <c r="L10" s="27" t="inlineStr">
         <is>
-          <t>-9%</t>
-        </is>
-      </c>
-      <c r="M10" s="26" t="inlineStr">
-        <is>
-          <t>-612bps</t>
-        </is>
-      </c>
-      <c r="N10" s="23" t="inlineStr">
-        <is>
-          <t>+55%</t>
+          <t>+161%</t>
+        </is>
+      </c>
+      <c r="M10" s="28" t="inlineStr">
+        <is>
+          <t>+519bps</t>
+        </is>
+      </c>
+      <c r="N10" s="24" t="inlineStr">
+        <is>
+          <t>+41%</t>
         </is>
       </c>
       <c r="O10" s="27" t="inlineStr">
         <is>
-          <t>-4%</t>
-        </is>
-      </c>
-      <c r="P10" s="26" t="inlineStr">
-        <is>
-          <t>-410bps</t>
+          <t>+89%</t>
+        </is>
+      </c>
+      <c r="P10" s="28" t="inlineStr">
+        <is>
+          <t>+356bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>6/28/2026</t>
+          <t>7/5/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>187265340</v>
+        <v>198331851</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>20773685</v>
+        <v>13762042</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.1109318200581058</v>
+        <v>0.06938896566845433</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>178427790</v>
+        <v>187715921</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>25667736</v>
+        <v>13578971</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.1438550351377439</v>
+        <v>0.07233787591197445</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>34322403</v>
+        <v>39155250</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>4555167</v>
+        <v>2644188</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.1327170186772762</v>
+        <v>0.06753086750818856</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>59305990</v>
+        <v>62287631</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>5238538</v>
+        <v>3223781</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.08833067283760039</v>
+        <v>0.05175635913974638</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>512508333</v>
+        <v>548797512</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>61849542</v>
+        <v>36510807</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.120680070971646</v>
+        <v>0.06652874002096423</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
-        <is>
-          <t>+306bps</t>
-        </is>
-      </c>
-      <c r="E12" s="29" t="inlineStr">
-        <is>
-          <t>+49%</t>
-        </is>
-      </c>
-      <c r="F12" s="30" t="inlineStr">
-        <is>
-          <t>+67%</t>
-        </is>
-      </c>
-      <c r="G12" s="31" t="inlineStr">
-        <is>
-          <t>+158bps</t>
-        </is>
-      </c>
-      <c r="H12" s="29" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="I12" s="30" t="inlineStr">
-        <is>
-          <t>+417%</t>
-        </is>
-      </c>
-      <c r="J12" s="31" t="inlineStr">
-        <is>
-          <t>+974bps</t>
-        </is>
-      </c>
-      <c r="K12" s="29" t="inlineStr">
-        <is>
-          <t>+73%</t>
-        </is>
-      </c>
-      <c r="L12" s="30" t="inlineStr">
-        <is>
-          <t>+100%</t>
-        </is>
-      </c>
-      <c r="M12" s="31" t="inlineStr">
-        <is>
-          <t>+117bps</t>
-        </is>
-      </c>
-      <c r="N12" s="29" t="inlineStr">
-        <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="O12" s="30" t="inlineStr">
-        <is>
-          <t>+86%</t>
-        </is>
-      </c>
-      <c r="P12" s="31" t="inlineStr">
-        <is>
-          <t>+255bps</t>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>+2%</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>-319bps</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>+1%</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="inlineStr">
+        <is>
+          <t>-407bps</t>
+        </is>
+      </c>
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>+60%</t>
+        </is>
+      </c>
+      <c r="I12" s="31" t="inlineStr">
+        <is>
+          <t>+20%</t>
+        </is>
+      </c>
+      <c r="J12" s="32" t="inlineStr">
+        <is>
+          <t>-223bps</t>
+        </is>
+      </c>
+      <c r="K12" s="30" t="inlineStr">
+        <is>
+          <t>+98%</t>
+        </is>
+      </c>
+      <c r="L12" s="33" t="inlineStr">
+        <is>
+          <t>-9%</t>
+        </is>
+      </c>
+      <c r="M12" s="32" t="inlineStr">
+        <is>
+          <t>-612bps</t>
+        </is>
+      </c>
+      <c r="N12" s="30" t="inlineStr">
+        <is>
+          <t>+55%</t>
+        </is>
+      </c>
+      <c r="O12" s="33" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="P12" s="32" t="inlineStr">
+        <is>
+          <t>-410bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Aug 13 20:49:05 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,18 +210,15 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -243,13 +240,16 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -264,10 +264,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -774,53 +771,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>8/2/2026</t>
+          <t>8/9/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>130246036</v>
+        <v>125731438</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>16204920</v>
+        <v>11195807</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.1244177596314716</v>
+        <v>0.08904540644798797</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>136855999</v>
+        <v>131288243</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>18214019</v>
+        <v>14045656</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.133088933865442</v>
+        <v>0.1069833496057983</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>33134991</v>
+        <v>25099261</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>2695236</v>
+        <v>3458247</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.08134108139640056</v>
+        <v>0.1377828215739101</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>43379501</v>
+        <v>48494523</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>5473675</v>
+        <v>4176190</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.126181142563166</v>
+        <v>0.08611673528575588</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>384761041</v>
+        <v>372916925</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>46532432</v>
+        <v>36677501</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.120938522983152</v>
+        <v>0.09835300717445312</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -831,264 +828,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
+          <t>+19%</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>-191bps</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>-129bps</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>+40%</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>+366bps</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
+          <t>+12%</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>-278bps</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
           <t>+18%</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>-58bps</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>+22%</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>-163bps</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>+23%</t>
-        </is>
-      </c>
-      <c r="I4" s="16" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>-559bps</t>
-        </is>
-      </c>
-      <c r="K4" s="17" t="inlineStr">
-        <is>
-          <t>-7%</t>
-        </is>
-      </c>
-      <c r="L4" s="16" t="inlineStr">
-        <is>
-          <t>-243%</t>
-        </is>
-      </c>
-      <c r="M4" s="18" t="inlineStr">
-        <is>
-          <t>+2082bps</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>+28%</t>
-        </is>
-      </c>
-      <c r="P4" s="18" t="inlineStr">
-        <is>
-          <t>+140bps</t>
+      <c r="O4" s="16" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>-121bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>7/26/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>121558881</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>8980474</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>0.0738775639107767</v>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>123109037</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>10499562</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>0.08528668776769004</v>
-      </c>
-      <c r="H5" s="20" t="n">
-        <v>24313828</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>2831499</v>
-      </c>
-      <c r="J5" s="22" t="n">
-        <v>0.1164563227147942</v>
-      </c>
-      <c r="K5" s="20" t="n">
-        <v>45125668</v>
-      </c>
-      <c r="L5" s="21" t="n">
-        <v>2828135</v>
-      </c>
-      <c r="M5" s="22" t="n">
-        <v>0.06267242404034883</v>
-      </c>
-      <c r="N5" s="20" t="n">
-        <v>354055496</v>
-      </c>
-      <c r="O5" s="21" t="n">
-        <v>27911568</v>
-      </c>
-      <c r="P5" s="22" t="n">
-        <v>0.0788338786301456</v>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>8/2/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>130246036</v>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>16204920</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>0.1244177596314716</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>136855999</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>18214019</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>0.133088933865442</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>33134991</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>2695236</v>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>0.08134108139640056</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>43379501</v>
+      </c>
+      <c r="L5" s="20" t="n">
+        <v>5473675</v>
+      </c>
+      <c r="M5" s="21" t="n">
+        <v>0.126181142563166</v>
+      </c>
+      <c r="N5" s="19" t="n">
+        <v>384761041</v>
+      </c>
+      <c r="O5" s="20" t="n">
+        <v>46532432</v>
+      </c>
+      <c r="P5" s="21" t="n">
+        <v>0.120938522983152</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>+6%</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>-28%</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>-347bps</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="inlineStr">
-        <is>
-          <t>+8%</t>
-        </is>
-      </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="G6" s="26" t="inlineStr">
-        <is>
-          <t>-186bps</t>
-        </is>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="I6" s="27" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>+18%</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>+13%</t>
         </is>
       </c>
-      <c r="J6" s="28" t="inlineStr">
-        <is>
-          <t>+76bps</t>
-        </is>
-      </c>
-      <c r="K6" s="24" t="inlineStr">
-        <is>
-          <t>+44%</t>
-        </is>
-      </c>
-      <c r="L6" s="25" t="inlineStr">
-        <is>
-          <t>-24%</t>
-        </is>
-      </c>
-      <c r="M6" s="26" t="inlineStr">
-        <is>
-          <t>-554bps</t>
-        </is>
-      </c>
-      <c r="N6" s="24" t="inlineStr">
-        <is>
-          <t>+8%</t>
-        </is>
-      </c>
-      <c r="O6" s="25" t="inlineStr">
-        <is>
-          <t>-20%</t>
-        </is>
-      </c>
-      <c r="P6" s="26" t="inlineStr">
-        <is>
-          <t>-273bps</t>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>-58bps</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>+22%</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>-163bps</t>
+        </is>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="I6" s="26" t="inlineStr">
+        <is>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="J6" s="25" t="inlineStr">
+        <is>
+          <t>-559bps</t>
+        </is>
+      </c>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t>-7%</t>
+        </is>
+      </c>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>-243%</t>
+        </is>
+      </c>
+      <c r="M6" s="28" t="inlineStr">
+        <is>
+          <t>+2082bps</t>
+        </is>
+      </c>
+      <c r="N6" s="23" t="inlineStr">
+        <is>
+          <t>+14%</t>
+        </is>
+      </c>
+      <c r="O6" s="24" t="inlineStr">
+        <is>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="P6" s="28" t="inlineStr">
+        <is>
+          <t>+140bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>7/19/2026</t>
+          <t>7/26/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>139807492</v>
+        <v>121558881</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>23125849</v>
+        <v>8980474</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.1654120867857354</v>
+        <v>0.0738775639107767</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>133999845</v>
+        <v>123109037</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>26554139</v>
+        <v>10499562</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1981654456391349</v>
+        <v>0.08528668776769004</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>29900329</v>
+        <v>24313828</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>4363449</v>
+        <v>2831499</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.1459331434112314</v>
+        <v>0.1164563227147942</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>48553128</v>
+        <v>45125668</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>4987561</v>
+        <v>2828135</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.1027237833162881</v>
+        <v>0.06267242404034883</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>396178246</v>
+        <v>354055496</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>63579445</v>
+        <v>27911568</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.1604819185352242</v>
+        <v>0.0788338786301456</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1099,264 +1096,264 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>+39%</t>
+          <t>+6%</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>+168%</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>+796bps</t>
+          <t>-28%</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>-347bps</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>+50%</t>
+          <t>+8%</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>+83%</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>+358bps</t>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>-186bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+78%</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>+96%</t>
-        </is>
-      </c>
-      <c r="J8" s="18" t="inlineStr">
-        <is>
-          <t>+137bps</t>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>+13%</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t>+76bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>+72%</t>
+          <t>+44%</t>
         </is>
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>+57%</t>
+          <t>-24%</t>
         </is>
       </c>
       <c r="M8" s="15" t="inlineStr">
         <is>
-          <t>-96bps</t>
+          <t>-554bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+49%</t>
+          <t>+8%</t>
         </is>
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="P8" s="18" t="inlineStr">
-        <is>
-          <t>+399bps</t>
+          <t>-20%</t>
+        </is>
+      </c>
+      <c r="P8" s="15" t="inlineStr">
+        <is>
+          <t>-273bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>7/12/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>165737601</v>
-      </c>
-      <c r="C9" s="21" t="n">
-        <v>23467231</v>
-      </c>
-      <c r="D9" s="22" t="n">
-        <v>0.1415926793823931</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>162520980</v>
-      </c>
-      <c r="F9" s="21" t="n">
-        <v>24960939</v>
-      </c>
-      <c r="G9" s="22" t="n">
-        <v>0.1535859493340491</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>34868855</v>
-      </c>
-      <c r="I9" s="21" t="n">
-        <v>4459574</v>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>0.1278956249065248</v>
-      </c>
-      <c r="K9" s="20" t="n">
-        <v>51411108</v>
-      </c>
-      <c r="L9" s="21" t="n">
-        <v>7470125</v>
-      </c>
-      <c r="M9" s="22" t="n">
-        <v>0.1453017701933209</v>
-      </c>
-      <c r="N9" s="20" t="n">
-        <v>464461727</v>
-      </c>
-      <c r="O9" s="21" t="n">
-        <v>65981611</v>
-      </c>
-      <c r="P9" s="22" t="n">
-        <v>0.1420603833736337</v>
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>7/19/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>139807492</v>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>23125849</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0.1654120867857354</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>133999845</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>26554139</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>0.1981654456391349</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>29900329</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>4363449</v>
+      </c>
+      <c r="J9" s="21" t="n">
+        <v>0.1459331434112314</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>48553128</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>4987561</v>
+      </c>
+      <c r="M9" s="21" t="n">
+        <v>0.1027237833162881</v>
+      </c>
+      <c r="N9" s="19" t="n">
+        <v>396178246</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <v>63579445</v>
+      </c>
+      <c r="P9" s="21" t="n">
+        <v>0.1604819185352242</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>+35%</t>
-        </is>
-      </c>
-      <c r="C10" s="27" t="inlineStr">
-        <is>
-          <t>+87%</t>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>+39%</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>+168%</t>
         </is>
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>+391bps</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="inlineStr">
-        <is>
-          <t>+65%</t>
+          <t>+796bps</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>+50%</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>+83%</t>
         </is>
       </c>
       <c r="G10" s="28" t="inlineStr">
         <is>
-          <t>+189bps</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="I10" s="27" t="inlineStr">
-        <is>
-          <t>+161%</t>
+          <t>+358bps</t>
+        </is>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>+78%</t>
+        </is>
+      </c>
+      <c r="I10" s="24" t="inlineStr">
+        <is>
+          <t>+96%</t>
         </is>
       </c>
       <c r="J10" s="28" t="inlineStr">
         <is>
-          <t>+520bps</t>
-        </is>
-      </c>
-      <c r="K10" s="24" t="inlineStr">
-        <is>
-          <t>+68%</t>
-        </is>
-      </c>
-      <c r="L10" s="27" t="inlineStr">
-        <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="M10" s="28" t="inlineStr">
-        <is>
-          <t>+519bps</t>
-        </is>
-      </c>
-      <c r="N10" s="24" t="inlineStr">
-        <is>
-          <t>+41%</t>
-        </is>
-      </c>
-      <c r="O10" s="27" t="inlineStr">
-        <is>
-          <t>+89%</t>
+          <t>+137bps</t>
+        </is>
+      </c>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>+72%</t>
+        </is>
+      </c>
+      <c r="L10" s="24" t="inlineStr">
+        <is>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="M10" s="25" t="inlineStr">
+        <is>
+          <t>-96bps</t>
+        </is>
+      </c>
+      <c r="N10" s="23" t="inlineStr">
+        <is>
+          <t>+49%</t>
+        </is>
+      </c>
+      <c r="O10" s="24" t="inlineStr">
+        <is>
+          <t>+98%</t>
         </is>
       </c>
       <c r="P10" s="28" t="inlineStr">
         <is>
-          <t>+356bps</t>
+          <t>+399bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>7/5/2026</t>
+          <t>7/12/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>198331851</v>
+        <v>165737601</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>13762042</v>
+        <v>23467231</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.06938896566845433</v>
+        <v>0.1415926793823931</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>187715921</v>
+        <v>162520980</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>13578971</v>
+        <v>24960939</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.07233787591197445</v>
+        <v>0.1535859493340491</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>39155250</v>
+        <v>34868855</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>2644188</v>
+        <v>4459574</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.06753086750818856</v>
+        <v>0.1278956249065248</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>62287631</v>
+        <v>51411108</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>3223781</v>
+        <v>7470125</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.05175635913974638</v>
+        <v>0.1453017701933209</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>548797512</v>
+        <v>464461727</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>36510807</v>
+        <v>65981611</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.06652874002096423</v>
+        <v>0.1420603833736337</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1367,77 +1364,77 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>+48%</t>
+          <t>+35%</t>
         </is>
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>+2%</t>
+          <t>+87%</t>
         </is>
       </c>
       <c r="D12" s="32" t="inlineStr">
         <is>
-          <t>-319bps</t>
+          <t>+391bps</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>+57%</t>
+          <t>+45%</t>
         </is>
       </c>
       <c r="F12" s="31" t="inlineStr">
         <is>
-          <t>+1%</t>
+          <t>+65%</t>
         </is>
       </c>
       <c r="G12" s="32" t="inlineStr">
         <is>
-          <t>-407bps</t>
+          <t>+189bps</t>
         </is>
       </c>
       <c r="H12" s="30" t="inlineStr">
         <is>
-          <t>+60%</t>
+          <t>+55%</t>
         </is>
       </c>
       <c r="I12" s="31" t="inlineStr">
         <is>
-          <t>+20%</t>
+          <t>+161%</t>
         </is>
       </c>
       <c r="J12" s="32" t="inlineStr">
         <is>
-          <t>-223bps</t>
+          <t>+520bps</t>
         </is>
       </c>
       <c r="K12" s="30" t="inlineStr">
         <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="L12" s="33" t="inlineStr">
-        <is>
-          <t>-9%</t>
+          <t>+68%</t>
+        </is>
+      </c>
+      <c r="L12" s="31" t="inlineStr">
+        <is>
+          <t>+161%</t>
         </is>
       </c>
       <c r="M12" s="32" t="inlineStr">
         <is>
-          <t>-612bps</t>
+          <t>+519bps</t>
         </is>
       </c>
       <c r="N12" s="30" t="inlineStr">
         <is>
-          <t>+55%</t>
-        </is>
-      </c>
-      <c r="O12" s="33" t="inlineStr">
-        <is>
-          <t>-4%</t>
+          <t>+41%</t>
+        </is>
+      </c>
+      <c r="O12" s="31" t="inlineStr">
+        <is>
+          <t>+89%</t>
         </is>
       </c>
       <c r="P12" s="32" t="inlineStr">
         <is>
-          <t>-410bps</t>
+          <t>+356bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Aug 20 14:40:16 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,51 +210,51 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -265,6 +265,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -771,53 +774,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>8/9/2026</t>
+          <t>8/16/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>125731438</v>
+        <v>139804782</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>11195807</v>
+        <v>14936414</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.08904540644798797</v>
+        <v>0.1068376473703167</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>131288243</v>
+        <v>128334482</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>14045656</v>
+        <v>16567440</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.1069833496057983</v>
+        <v>0.1290957795738794</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>25099261</v>
+        <v>26211607</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>3458247</v>
+        <v>3989974</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.1377828215739101</v>
+        <v>0.1522216474556482</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>48494523</v>
+        <v>43618315</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>4176190</v>
+        <v>4332991</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.08611673528575588</v>
+        <v>0.09933879839237256</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>372916925</v>
+        <v>380789208</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>36677501</v>
+        <v>44525193</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.09835300717445312</v>
+        <v>0.1169287155848177</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -828,264 +831,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+19%</t>
+          <t>+14%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>-2%</t>
+          <t>+38%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>-191bps</t>
+          <t>+182bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+16%</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>+3%</t>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>+17%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>-129bps</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="I4" s="16" t="inlineStr">
-        <is>
-          <t>+40%</t>
-        </is>
-      </c>
-      <c r="J4" s="17" t="inlineStr">
-        <is>
-          <t>+366bps</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>+48%</t>
-        </is>
-      </c>
-      <c r="L4" s="16" t="inlineStr">
-        <is>
-          <t>+12%</t>
+          <t>+80bps</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>-1%</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>+590bps</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="inlineStr">
+        <is>
+          <t>-70%</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>+61%</t>
         </is>
       </c>
       <c r="M4" s="15" t="inlineStr">
         <is>
-          <t>-278bps</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>+18%</t>
-        </is>
-      </c>
-      <c r="O4" s="16" t="inlineStr">
-        <is>
-          <t>+5%</t>
+          <t>+811bps</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>-17%</t>
+        </is>
+      </c>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>+34%</t>
         </is>
       </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
-          <t>-121bps</t>
+          <t>+441bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>8/2/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>130246036</v>
-      </c>
-      <c r="C5" s="20" t="n">
-        <v>16204920</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>0.1244177596314716</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>136855999</v>
-      </c>
-      <c r="F5" s="20" t="n">
-        <v>18214019</v>
-      </c>
-      <c r="G5" s="21" t="n">
-        <v>0.133088933865442</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>33134991</v>
-      </c>
-      <c r="I5" s="20" t="n">
-        <v>2695236</v>
-      </c>
-      <c r="J5" s="21" t="n">
-        <v>0.08134108139640056</v>
-      </c>
-      <c r="K5" s="19" t="n">
-        <v>43379501</v>
-      </c>
-      <c r="L5" s="20" t="n">
-        <v>5473675</v>
-      </c>
-      <c r="M5" s="21" t="n">
-        <v>0.126181142563166</v>
-      </c>
-      <c r="N5" s="19" t="n">
-        <v>384761041</v>
-      </c>
-      <c r="O5" s="20" t="n">
-        <v>46532432</v>
-      </c>
-      <c r="P5" s="21" t="n">
-        <v>0.120938522983152</v>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>8/9/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>125731438</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>11195807</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>0.08904540644798797</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>131288243</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>14045656</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>0.1069833496057983</v>
+      </c>
+      <c r="H5" s="18" t="n">
+        <v>25099261</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>3458247</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <v>0.1377828215739101</v>
+      </c>
+      <c r="K5" s="18" t="n">
+        <v>48494523</v>
+      </c>
+      <c r="L5" s="19" t="n">
+        <v>4176190</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>0.08611673528575588</v>
+      </c>
+      <c r="N5" s="18" t="n">
+        <v>372916925</v>
+      </c>
+      <c r="O5" s="19" t="n">
+        <v>36677501</v>
+      </c>
+      <c r="P5" s="20" t="n">
+        <v>0.09835300717445312</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>+19%</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>-191bps</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>-129bps</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>+40%</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>+366bps</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="L6" s="25" t="inlineStr">
+        <is>
+          <t>+12%</t>
+        </is>
+      </c>
+      <c r="M6" s="24" t="inlineStr">
+        <is>
+          <t>-278bps</t>
+        </is>
+      </c>
+      <c r="N6" s="22" t="inlineStr">
         <is>
           <t>+18%</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>-58bps</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>+22%</t>
-        </is>
-      </c>
-      <c r="F6" s="24" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>-163bps</t>
-        </is>
-      </c>
-      <c r="H6" s="23" t="inlineStr">
-        <is>
-          <t>+23%</t>
-        </is>
-      </c>
-      <c r="I6" s="26" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="J6" s="25" t="inlineStr">
-        <is>
-          <t>-559bps</t>
-        </is>
-      </c>
-      <c r="K6" s="27" t="inlineStr">
-        <is>
-          <t>-7%</t>
-        </is>
-      </c>
-      <c r="L6" s="26" t="inlineStr">
-        <is>
-          <t>-243%</t>
-        </is>
-      </c>
-      <c r="M6" s="28" t="inlineStr">
-        <is>
-          <t>+2082bps</t>
-        </is>
-      </c>
-      <c r="N6" s="23" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="O6" s="24" t="inlineStr">
-        <is>
-          <t>+28%</t>
-        </is>
-      </c>
-      <c r="P6" s="28" t="inlineStr">
-        <is>
-          <t>+140bps</t>
+      <c r="O6" s="25" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="P6" s="24" t="inlineStr">
+        <is>
+          <t>-121bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>7/26/2026</t>
+          <t>8/2/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>121558881</v>
+        <v>130246036</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>8980474</v>
+        <v>16204920</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.0738775639107767</v>
+        <v>0.1244177596314716</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>123109037</v>
+        <v>136855999</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>10499562</v>
+        <v>18214019</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.08528668776769004</v>
+        <v>0.133088933865442</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>24313828</v>
+        <v>33134991</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>2831499</v>
+        <v>2695236</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.1164563227147942</v>
+        <v>0.08134108139640056</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>45125668</v>
+        <v>43379501</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>2828135</v>
+        <v>5473675</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.06267242404034883</v>
+        <v>0.126181142563166</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>354055496</v>
+        <v>384761041</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>27911568</v>
+        <v>46532432</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.0788338786301456</v>
+        <v>0.120938522983152</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1096,264 +1099,264 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>+6%</t>
+          <t>+18%</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>-28%</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>-347bps</t>
+          <t>+13%</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>-58bps</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>+8%</t>
+          <t>+22%</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>-186bps</t>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>-163bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="J8" s="17" t="inlineStr">
-        <is>
-          <t>+76bps</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>+44%</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr">
-        <is>
-          <t>-24%</t>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="I8" s="28" t="inlineStr">
+        <is>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="J8" s="27" t="inlineStr">
+        <is>
+          <t>-559bps</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>-7%</t>
+        </is>
+      </c>
+      <c r="L8" s="28" t="inlineStr">
+        <is>
+          <t>-243%</t>
         </is>
       </c>
       <c r="M8" s="15" t="inlineStr">
         <is>
-          <t>-554bps</t>
+          <t>+2082bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+8%</t>
+          <t>+14%</t>
         </is>
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>-20%</t>
+          <t>+28%</t>
         </is>
       </c>
       <c r="P8" s="15" t="inlineStr">
         <is>
-          <t>-273bps</t>
+          <t>+140bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>7/19/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>139807492</v>
-      </c>
-      <c r="C9" s="20" t="n">
-        <v>23125849</v>
-      </c>
-      <c r="D9" s="21" t="n">
-        <v>0.1654120867857354</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>133999845</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>26554139</v>
-      </c>
-      <c r="G9" s="21" t="n">
-        <v>0.1981654456391349</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>29900329</v>
-      </c>
-      <c r="I9" s="20" t="n">
-        <v>4363449</v>
-      </c>
-      <c r="J9" s="21" t="n">
-        <v>0.1459331434112314</v>
-      </c>
-      <c r="K9" s="19" t="n">
-        <v>48553128</v>
-      </c>
-      <c r="L9" s="20" t="n">
-        <v>4987561</v>
-      </c>
-      <c r="M9" s="21" t="n">
-        <v>0.1027237833162881</v>
-      </c>
-      <c r="N9" s="19" t="n">
-        <v>396178246</v>
-      </c>
-      <c r="O9" s="20" t="n">
-        <v>63579445</v>
-      </c>
-      <c r="P9" s="21" t="n">
-        <v>0.1604819185352242</v>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>7/26/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>121558881</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>8980474</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>0.0738775639107767</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>123109037</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>10499562</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>0.08528668776769004</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>24313828</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>2831499</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>0.1164563227147942</v>
+      </c>
+      <c r="K9" s="18" t="n">
+        <v>45125668</v>
+      </c>
+      <c r="L9" s="19" t="n">
+        <v>2828135</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <v>0.06267242404034883</v>
+      </c>
+      <c r="N9" s="18" t="n">
+        <v>354055496</v>
+      </c>
+      <c r="O9" s="19" t="n">
+        <v>27911568</v>
+      </c>
+      <c r="P9" s="20" t="n">
+        <v>0.0788338786301456</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>+39%</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>+168%</t>
-        </is>
-      </c>
-      <c r="D10" s="28" t="inlineStr">
-        <is>
-          <t>+796bps</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>+50%</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr">
-        <is>
-          <t>+83%</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr">
-        <is>
-          <t>+358bps</t>
-        </is>
-      </c>
-      <c r="H10" s="23" t="inlineStr">
-        <is>
-          <t>+78%</t>
-        </is>
-      </c>
-      <c r="I10" s="24" t="inlineStr">
-        <is>
-          <t>+96%</t>
-        </is>
-      </c>
-      <c r="J10" s="28" t="inlineStr">
-        <is>
-          <t>+137bps</t>
-        </is>
-      </c>
-      <c r="K10" s="23" t="inlineStr">
-        <is>
-          <t>+72%</t>
-        </is>
-      </c>
-      <c r="L10" s="24" t="inlineStr">
-        <is>
-          <t>+57%</t>
-        </is>
-      </c>
-      <c r="M10" s="25" t="inlineStr">
-        <is>
-          <t>-96bps</t>
-        </is>
-      </c>
-      <c r="N10" s="23" t="inlineStr">
-        <is>
-          <t>+49%</t>
-        </is>
-      </c>
-      <c r="O10" s="24" t="inlineStr">
-        <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="P10" s="28" t="inlineStr">
-        <is>
-          <t>+399bps</t>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>+6%</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>-28%</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>-347bps</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>-186bps</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>+13%</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t>+76bps</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="inlineStr">
+        <is>
+          <t>+44%</t>
+        </is>
+      </c>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>-24%</t>
+        </is>
+      </c>
+      <c r="M10" s="24" t="inlineStr">
+        <is>
+          <t>-554bps</t>
+        </is>
+      </c>
+      <c r="N10" s="22" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>-20%</t>
+        </is>
+      </c>
+      <c r="P10" s="24" t="inlineStr">
+        <is>
+          <t>-273bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>7/12/2026</t>
+          <t>7/19/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>165737601</v>
+        <v>139807492</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>23467231</v>
+        <v>23125849</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.1415926793823931</v>
+        <v>0.1654120867857354</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>162520980</v>
+        <v>133999845</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>24960939</v>
+        <v>26554139</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.1535859493340491</v>
+        <v>0.1981654456391349</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>34868855</v>
+        <v>29900329</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>4459574</v>
+        <v>4363449</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.1278956249065248</v>
+        <v>0.1459331434112314</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>51411108</v>
+        <v>48553128</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>7470125</v>
+        <v>4987561</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.1453017701933209</v>
+        <v>0.1027237833162881</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>464461727</v>
+        <v>396178246</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>65981611</v>
+        <v>63579445</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.1420603833736337</v>
+        <v>0.1604819185352242</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1364,77 +1367,77 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>+35%</t>
+          <t>+39%</t>
         </is>
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>+87%</t>
+          <t>+168%</t>
         </is>
       </c>
       <c r="D12" s="32" t="inlineStr">
         <is>
-          <t>+391bps</t>
+          <t>+796bps</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>+45%</t>
+          <t>+50%</t>
         </is>
       </c>
       <c r="F12" s="31" t="inlineStr">
         <is>
-          <t>+65%</t>
+          <t>+83%</t>
         </is>
       </c>
       <c r="G12" s="32" t="inlineStr">
         <is>
-          <t>+189bps</t>
+          <t>+358bps</t>
         </is>
       </c>
       <c r="H12" s="30" t="inlineStr">
         <is>
-          <t>+55%</t>
+          <t>+78%</t>
         </is>
       </c>
       <c r="I12" s="31" t="inlineStr">
         <is>
-          <t>+161%</t>
+          <t>+96%</t>
         </is>
       </c>
       <c r="J12" s="32" t="inlineStr">
         <is>
-          <t>+520bps</t>
+          <t>+137bps</t>
         </is>
       </c>
       <c r="K12" s="30" t="inlineStr">
         <is>
-          <t>+68%</t>
+          <t>+72%</t>
         </is>
       </c>
       <c r="L12" s="31" t="inlineStr">
         <is>
-          <t>+161%</t>
-        </is>
-      </c>
-      <c r="M12" s="32" t="inlineStr">
-        <is>
-          <t>+519bps</t>
+          <t>+57%</t>
+        </is>
+      </c>
+      <c r="M12" s="33" t="inlineStr">
+        <is>
+          <t>-96bps</t>
         </is>
       </c>
       <c r="N12" s="30" t="inlineStr">
         <is>
-          <t>+41%</t>
+          <t>+49%</t>
         </is>
       </c>
       <c r="O12" s="31" t="inlineStr">
         <is>
-          <t>+89%</t>
+          <t>+98%</t>
         </is>
       </c>
       <c r="P12" s="32" t="inlineStr">
         <is>
-          <t>+356bps</t>
+          <t>+399bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Aug 27 17:59:25 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,15 +210,21 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -237,37 +243,37 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -774,53 +780,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>8/16/2026</t>
+          <t>8/23/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>139804782</v>
+        <v>137507207</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>14936414</v>
+        <v>10643451</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.1068376473703167</v>
+        <v>0.07740285932794781</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>128334482</v>
+        <v>132060011</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>16567440</v>
+        <v>10710519</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.1290957795738794</v>
+        <v>0.08110342350342527</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>26211607</v>
+        <v>24881322</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>3989974</v>
+        <v>1911178</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.1522216474556482</v>
+        <v>0.07681175461657544</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>43618315</v>
+        <v>47701558</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>4332991</v>
+        <v>3476356</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.09933879839237256</v>
+        <v>0.07287720036314117</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>380789208</v>
+        <v>381646903</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>44525193</v>
+        <v>30506351</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.1169287155848177</v>
+        <v>0.07993344308626553</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -831,264 +837,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+14%</t>
+          <t>+4%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>+38%</t>
+          <t>-31%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>+182bps</t>
+          <t>-395bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+9%</t>
+          <t>+5%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>+17%</t>
+          <t>-4%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>+80bps</t>
+          <t>-78bps</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-11%</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>+61%</t>
+          <t>-36%</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>+590bps</t>
+          <t>-301bps</t>
         </is>
       </c>
       <c r="K4" s="16" t="inlineStr">
         <is>
-          <t>-70%</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>+811bps</t>
+          <t>-78%</t>
+        </is>
+      </c>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>+688%</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>+708bps</t>
         </is>
       </c>
       <c r="N4" s="16" t="inlineStr">
         <is>
-          <t>-17%</t>
+          <t>-30%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>+34%</t>
-        </is>
-      </c>
-      <c r="P4" s="15" t="inlineStr">
-        <is>
-          <t>+441bps</t>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="P4" s="18" t="inlineStr">
+        <is>
+          <t>+170bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>8/9/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="n">
-        <v>125731438</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>11195807</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.08904540644798797</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>131288243</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>14045656</v>
-      </c>
-      <c r="G5" s="20" t="n">
-        <v>0.1069833496057983</v>
-      </c>
-      <c r="H5" s="18" t="n">
-        <v>25099261</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>3458247</v>
-      </c>
-      <c r="J5" s="20" t="n">
-        <v>0.1377828215739101</v>
-      </c>
-      <c r="K5" s="18" t="n">
-        <v>48494523</v>
-      </c>
-      <c r="L5" s="19" t="n">
-        <v>4176190</v>
-      </c>
-      <c r="M5" s="20" t="n">
-        <v>0.08611673528575588</v>
-      </c>
-      <c r="N5" s="18" t="n">
-        <v>372916925</v>
-      </c>
-      <c r="O5" s="19" t="n">
-        <v>36677501</v>
-      </c>
-      <c r="P5" s="20" t="n">
-        <v>0.09835300717445312</v>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>8/16/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>139804782</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>14936414</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>0.1068376473703167</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>128334482</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>16567440</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.1290957795738794</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>26211607</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>3989974</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.1522216474556482</v>
+      </c>
+      <c r="K5" s="20" t="n">
+        <v>43618315</v>
+      </c>
+      <c r="L5" s="21" t="n">
+        <v>4332991</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.09933879839237256</v>
+      </c>
+      <c r="N5" s="20" t="n">
+        <v>380789208</v>
+      </c>
+      <c r="O5" s="21" t="n">
+        <v>44525193</v>
+      </c>
+      <c r="P5" s="22" t="n">
+        <v>0.1169287155848177</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>+19%</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>-2%</t>
-        </is>
-      </c>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>-191bps</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>+16%</t>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>+14%</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>+182bps</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>+9%</t>
         </is>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="G6" s="24" t="inlineStr">
-        <is>
-          <t>-129bps</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>+3%</t>
+          <t>+17%</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>+80bps</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>-1%</t>
         </is>
       </c>
       <c r="I6" s="25" t="inlineStr">
         <is>
-          <t>+40%</t>
+          <t>+61%</t>
         </is>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
-          <t>+366bps</t>
-        </is>
-      </c>
-      <c r="K6" s="22" t="inlineStr">
-        <is>
-          <t>+48%</t>
+          <t>+590bps</t>
+        </is>
+      </c>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t>-70%</t>
         </is>
       </c>
       <c r="L6" s="25" t="inlineStr">
         <is>
-          <t>+12%</t>
-        </is>
-      </c>
-      <c r="M6" s="24" t="inlineStr">
-        <is>
-          <t>-278bps</t>
-        </is>
-      </c>
-      <c r="N6" s="22" t="inlineStr">
-        <is>
-          <t>+18%</t>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="M6" s="26" t="inlineStr">
+        <is>
+          <t>+811bps</t>
+        </is>
+      </c>
+      <c r="N6" s="27" t="inlineStr">
+        <is>
+          <t>-17%</t>
         </is>
       </c>
       <c r="O6" s="25" t="inlineStr">
         <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="P6" s="24" t="inlineStr">
-        <is>
-          <t>-121bps</t>
+          <t>+34%</t>
+        </is>
+      </c>
+      <c r="P6" s="26" t="inlineStr">
+        <is>
+          <t>+441bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>8/2/2026</t>
+          <t>8/9/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>130246036</v>
+        <v>125731438</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>16204920</v>
+        <v>11195807</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.1244177596314716</v>
+        <v>0.08904540644798797</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>136855999</v>
+        <v>131288243</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>18214019</v>
+        <v>14045656</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.133088933865442</v>
+        <v>0.1069833496057983</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>33134991</v>
+        <v>25099261</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>2695236</v>
+        <v>3458247</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.08134108139640056</v>
+        <v>0.1377828215739101</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>43379501</v>
+        <v>48494523</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>5473675</v>
+        <v>4176190</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.126181142563166</v>
+        <v>0.08611673528575588</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>384761041</v>
+        <v>372916925</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>46532432</v>
+        <v>36677501</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.120938522983152</v>
+        <v>0.09835300717445312</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1099,345 +1105,345 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
+          <t>+19%</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>-191bps</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>-129bps</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>+40%</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>+366bps</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>+12%</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>-278bps</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
           <t>+18%</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>-58bps</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>+22%</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="G8" s="27" t="inlineStr">
-        <is>
-          <t>-163bps</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>+23%</t>
-        </is>
-      </c>
-      <c r="I8" s="28" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="J8" s="27" t="inlineStr">
-        <is>
-          <t>-559bps</t>
-        </is>
-      </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>-7%</t>
-        </is>
-      </c>
-      <c r="L8" s="28" t="inlineStr">
-        <is>
-          <t>-243%</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>+2082bps</t>
-        </is>
-      </c>
-      <c r="N8" s="13" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="O8" s="14" t="inlineStr">
-        <is>
-          <t>+28%</t>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>+5%</t>
         </is>
       </c>
       <c r="P8" s="15" t="inlineStr">
         <is>
-          <t>+140bps</t>
+          <t>-121bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>7/26/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>121558881</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>8980474</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0.0738775639107767</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>123109037</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>10499562</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>0.08528668776769004</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>24313828</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>2831499</v>
-      </c>
-      <c r="J9" s="20" t="n">
-        <v>0.1164563227147942</v>
-      </c>
-      <c r="K9" s="18" t="n">
-        <v>45125668</v>
-      </c>
-      <c r="L9" s="19" t="n">
-        <v>2828135</v>
-      </c>
-      <c r="M9" s="20" t="n">
-        <v>0.06267242404034883</v>
-      </c>
-      <c r="N9" s="18" t="n">
-        <v>354055496</v>
-      </c>
-      <c r="O9" s="19" t="n">
-        <v>27911568</v>
-      </c>
-      <c r="P9" s="20" t="n">
-        <v>0.0788338786301456</v>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>8/2/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>130246036</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>16204920</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.1244177596314716</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>136855999</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>18214019</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>0.133088933865442</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>33134991</v>
+      </c>
+      <c r="I9" s="21" t="n">
+        <v>2695236</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.08134108139640056</v>
+      </c>
+      <c r="K9" s="20" t="n">
+        <v>43379501</v>
+      </c>
+      <c r="L9" s="21" t="n">
+        <v>5473675</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>0.126181142563166</v>
+      </c>
+      <c r="N9" s="20" t="n">
+        <v>384761041</v>
+      </c>
+      <c r="O9" s="21" t="n">
+        <v>46532432</v>
+      </c>
+      <c r="P9" s="22" t="n">
+        <v>0.120938522983152</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>+6%</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>-28%</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>-347bps</t>
-        </is>
-      </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>+8%</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="G10" s="24" t="inlineStr">
-        <is>
-          <t>-186bps</t>
-        </is>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="I10" s="25" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>+18%</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>+13%</t>
         </is>
       </c>
-      <c r="J10" s="26" t="inlineStr">
-        <is>
-          <t>+76bps</t>
-        </is>
-      </c>
-      <c r="K10" s="22" t="inlineStr">
-        <is>
-          <t>+44%</t>
-        </is>
-      </c>
-      <c r="L10" s="23" t="inlineStr">
-        <is>
-          <t>-24%</t>
-        </is>
-      </c>
-      <c r="M10" s="24" t="inlineStr">
-        <is>
-          <t>-554bps</t>
-        </is>
-      </c>
-      <c r="N10" s="22" t="inlineStr">
-        <is>
-          <t>+8%</t>
-        </is>
-      </c>
-      <c r="O10" s="23" t="inlineStr">
-        <is>
-          <t>-20%</t>
-        </is>
-      </c>
-      <c r="P10" s="24" t="inlineStr">
-        <is>
-          <t>-273bps</t>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>-58bps</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>+22%</t>
+        </is>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>-163bps</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="inlineStr">
+        <is>
+          <t>-559bps</t>
+        </is>
+      </c>
+      <c r="K10" s="27" t="inlineStr">
+        <is>
+          <t>-7%</t>
+        </is>
+      </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>-243%</t>
+        </is>
+      </c>
+      <c r="M10" s="26" t="inlineStr">
+        <is>
+          <t>+2082bps</t>
+        </is>
+      </c>
+      <c r="N10" s="24" t="inlineStr">
+        <is>
+          <t>+14%</t>
+        </is>
+      </c>
+      <c r="O10" s="25" t="inlineStr">
+        <is>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="P10" s="26" t="inlineStr">
+        <is>
+          <t>+140bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>7/19/2026</t>
+          <t>7/26/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>139807492</v>
+        <v>121558881</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>23125849</v>
+        <v>8980474</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.1654120867857354</v>
+        <v>0.0738775639107767</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>133999845</v>
+        <v>123109037</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>26554139</v>
+        <v>10499562</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.1981654456391349</v>
+        <v>0.08528668776769004</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>29900329</v>
+        <v>24313828</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>4363449</v>
+        <v>2831499</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.1459331434112314</v>
+        <v>0.1164563227147942</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>48553128</v>
+        <v>45125668</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>4987561</v>
+        <v>2828135</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.1027237833162881</v>
+        <v>0.06267242404034883</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>396178246</v>
+        <v>354055496</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>63579445</v>
+        <v>27911568</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.1604819185352242</v>
+        <v>0.0788338786301456</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>+39%</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>+168%</t>
-        </is>
-      </c>
-      <c r="D12" s="32" t="inlineStr">
-        <is>
-          <t>+796bps</t>
-        </is>
-      </c>
-      <c r="E12" s="30" t="inlineStr">
-        <is>
-          <t>+50%</t>
-        </is>
-      </c>
-      <c r="F12" s="31" t="inlineStr">
-        <is>
-          <t>+83%</t>
-        </is>
-      </c>
-      <c r="G12" s="32" t="inlineStr">
-        <is>
-          <t>+358bps</t>
-        </is>
-      </c>
-      <c r="H12" s="30" t="inlineStr">
-        <is>
-          <t>+78%</t>
-        </is>
-      </c>
-      <c r="I12" s="31" t="inlineStr">
-        <is>
-          <t>+96%</t>
-        </is>
-      </c>
-      <c r="J12" s="32" t="inlineStr">
-        <is>
-          <t>+137bps</t>
-        </is>
-      </c>
-      <c r="K12" s="30" t="inlineStr">
-        <is>
-          <t>+72%</t>
-        </is>
-      </c>
-      <c r="L12" s="31" t="inlineStr">
-        <is>
-          <t>+57%</t>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>+6%</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>-28%</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>-347bps</t>
+        </is>
+      </c>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>-186bps</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="I12" s="34" t="inlineStr">
+        <is>
+          <t>+13%</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>+76bps</t>
+        </is>
+      </c>
+      <c r="K12" s="31" t="inlineStr">
+        <is>
+          <t>+44%</t>
+        </is>
+      </c>
+      <c r="L12" s="32" t="inlineStr">
+        <is>
+          <t>-24%</t>
         </is>
       </c>
       <c r="M12" s="33" t="inlineStr">
         <is>
-          <t>-96bps</t>
-        </is>
-      </c>
-      <c r="N12" s="30" t="inlineStr">
-        <is>
-          <t>+49%</t>
-        </is>
-      </c>
-      <c r="O12" s="31" t="inlineStr">
-        <is>
-          <t>+98%</t>
-        </is>
-      </c>
-      <c r="P12" s="32" t="inlineStr">
-        <is>
-          <t>+399bps</t>
+          <t>-554bps</t>
+        </is>
+      </c>
+      <c r="N12" s="31" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="O12" s="32" t="inlineStr">
+        <is>
+          <t>-20%</t>
+        </is>
+      </c>
+      <c r="P12" s="33" t="inlineStr">
+        <is>
+          <t>-273bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Fri Sep  4 15:20:45 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -52,12 +52,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,70 +210,73 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -780,53 +783,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>8/23/2026</t>
+          <t>8/30/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>137507207</v>
+        <v>149527600</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>10643451</v>
+        <v>12079306</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.07740285932794781</v>
+        <v>0.08078311963811363</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>132060011</v>
+        <v>146777768</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>10710519</v>
+        <v>15874317</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.08110342350342527</v>
+        <v>0.1081520515320821</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>24881322</v>
+        <v>29155390</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>1911178</v>
+        <v>2727869</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.07681175461657544</v>
+        <v>0.09356311131492324</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>47701558</v>
+        <v>52848942</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>3476356</v>
+        <v>5061346</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.07287720036314117</v>
+        <v>0.09577005344780601</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>381646903</v>
+        <v>406173189</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>30506351</v>
+        <v>38184969</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.07993344308626553</v>
+        <v>0.09401154483512696</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -837,264 +840,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>+4%</t>
+          <t>-10%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>-31%</t>
+          <t>-39%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>-395bps</t>
+          <t>-392bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>+5%</t>
+          <t>-4%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>-4%</t>
+          <t>-27%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>-78bps</t>
-        </is>
-      </c>
-      <c r="H4" s="16" t="inlineStr">
-        <is>
-          <t>-11%</t>
+          <t>-338bps</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>-25%</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>-36%</t>
+          <t>-37%</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>-301bps</t>
-        </is>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>-78%</t>
-        </is>
-      </c>
-      <c r="L4" s="17" t="inlineStr">
-        <is>
-          <t>+688%</t>
-        </is>
-      </c>
-      <c r="M4" s="18" t="inlineStr">
-        <is>
-          <t>+708bps</t>
-        </is>
-      </c>
-      <c r="N4" s="16" t="inlineStr">
-        <is>
-          <t>-30%</t>
+          <t>-186bps</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>-64%</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>-66%</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>-57bps</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>-27%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="P4" s="18" t="inlineStr">
-        <is>
-          <t>+170bps</t>
+          <t>-43%</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>-254bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>8/16/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>139804782</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>14936414</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>0.1068376473703167</v>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>128334482</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>16567440</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>0.1290957795738794</v>
-      </c>
-      <c r="H5" s="20" t="n">
-        <v>26211607</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>3989974</v>
-      </c>
-      <c r="J5" s="22" t="n">
-        <v>0.1522216474556482</v>
-      </c>
-      <c r="K5" s="20" t="n">
-        <v>43618315</v>
-      </c>
-      <c r="L5" s="21" t="n">
-        <v>4332991</v>
-      </c>
-      <c r="M5" s="22" t="n">
-        <v>0.09933879839237256</v>
-      </c>
-      <c r="N5" s="20" t="n">
-        <v>380789208</v>
-      </c>
-      <c r="O5" s="21" t="n">
-        <v>44525193</v>
-      </c>
-      <c r="P5" s="22" t="n">
-        <v>0.1169287155848177</v>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>8/23/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>137507207</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>10643451</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0.07740285932794781</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>132060011</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>10710519</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>0.08110342350342527</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>24881322</v>
+      </c>
+      <c r="I5" s="18" t="n">
+        <v>1911178</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>0.07681175461657544</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>47701558</v>
+      </c>
+      <c r="L5" s="18" t="n">
+        <v>3476356</v>
+      </c>
+      <c r="M5" s="19" t="n">
+        <v>0.07287720036314117</v>
+      </c>
+      <c r="N5" s="17" t="n">
+        <v>381646903</v>
+      </c>
+      <c r="O5" s="18" t="n">
+        <v>30506351</v>
+      </c>
+      <c r="P5" s="19" t="n">
+        <v>0.07993344308626553</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>+182bps</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>+17%</t>
-        </is>
-      </c>
-      <c r="G6" s="26" t="inlineStr">
-        <is>
-          <t>+80bps</t>
-        </is>
-      </c>
-      <c r="H6" s="27" t="inlineStr">
-        <is>
-          <t>-1%</t>
-        </is>
-      </c>
-      <c r="I6" s="25" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="J6" s="26" t="inlineStr">
-        <is>
-          <t>+590bps</t>
-        </is>
-      </c>
-      <c r="K6" s="27" t="inlineStr">
-        <is>
-          <t>-70%</t>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>-31%</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>-395bps</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>-78bps</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>-36%</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>-301bps</t>
+        </is>
+      </c>
+      <c r="K6" s="24" t="inlineStr">
+        <is>
+          <t>-78%</t>
         </is>
       </c>
       <c r="L6" s="25" t="inlineStr">
         <is>
-          <t>+61%</t>
+          <t>+688%</t>
         </is>
       </c>
       <c r="M6" s="26" t="inlineStr">
         <is>
-          <t>+811bps</t>
-        </is>
-      </c>
-      <c r="N6" s="27" t="inlineStr">
-        <is>
-          <t>-17%</t>
-        </is>
-      </c>
-      <c r="O6" s="25" t="inlineStr">
-        <is>
-          <t>+34%</t>
+          <t>+708bps</t>
+        </is>
+      </c>
+      <c r="N6" s="24" t="inlineStr">
+        <is>
+          <t>-30%</t>
+        </is>
+      </c>
+      <c r="O6" s="22" t="inlineStr">
+        <is>
+          <t>-11%</t>
         </is>
       </c>
       <c r="P6" s="26" t="inlineStr">
         <is>
-          <t>+441bps</t>
+          <t>+170bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>8/9/2026</t>
+          <t>8/16/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>125731438</v>
+        <v>139804782</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>11195807</v>
+        <v>14936414</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.08904540644798797</v>
+        <v>0.1068376473703167</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>131288243</v>
+        <v>128334482</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>14045656</v>
+        <v>16567440</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1069833496057983</v>
+        <v>0.1290957795738794</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>25099261</v>
+        <v>26211607</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>3458247</v>
+        <v>3989974</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.1377828215739101</v>
+        <v>0.1522216474556482</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>48494523</v>
+        <v>43618315</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>4176190</v>
+        <v>4332991</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.08611673528575588</v>
+        <v>0.09933879839237256</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>372916925</v>
+        <v>380789208</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>36677501</v>
+        <v>44525193</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.09835300717445312</v>
+        <v>0.1169287155848177</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1103,266 +1106,266 @@
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>+19%</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>-2%</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>-191bps</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>+16%</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>-129bps</t>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>+14%</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>+182bps</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>+17%</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>+80bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="I8" s="17" t="inlineStr">
-        <is>
-          <t>+40%</t>
-        </is>
-      </c>
-      <c r="J8" s="18" t="inlineStr">
-        <is>
-          <t>+366bps</t>
+          <t>-1%</t>
+        </is>
+      </c>
+      <c r="I8" s="28" t="inlineStr">
+        <is>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>+590bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>+48%</t>
-        </is>
-      </c>
-      <c r="L8" s="17" t="inlineStr">
-        <is>
-          <t>+12%</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>-278bps</t>
+          <t>-70%</t>
+        </is>
+      </c>
+      <c r="L8" s="28" t="inlineStr">
+        <is>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="M8" s="29" t="inlineStr">
+        <is>
+          <t>+811bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>+18%</t>
-        </is>
-      </c>
-      <c r="O8" s="17" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="P8" s="15" t="inlineStr">
-        <is>
-          <t>-121bps</t>
+          <t>-17%</t>
+        </is>
+      </c>
+      <c r="O8" s="28" t="inlineStr">
+        <is>
+          <t>+34%</t>
+        </is>
+      </c>
+      <c r="P8" s="29" t="inlineStr">
+        <is>
+          <t>+441bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>8/2/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>130246036</v>
-      </c>
-      <c r="C9" s="21" t="n">
-        <v>16204920</v>
-      </c>
-      <c r="D9" s="22" t="n">
-        <v>0.1244177596314716</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>136855999</v>
-      </c>
-      <c r="F9" s="21" t="n">
-        <v>18214019</v>
-      </c>
-      <c r="G9" s="22" t="n">
-        <v>0.133088933865442</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>33134991</v>
-      </c>
-      <c r="I9" s="21" t="n">
-        <v>2695236</v>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>0.08134108139640056</v>
-      </c>
-      <c r="K9" s="20" t="n">
-        <v>43379501</v>
-      </c>
-      <c r="L9" s="21" t="n">
-        <v>5473675</v>
-      </c>
-      <c r="M9" s="22" t="n">
-        <v>0.126181142563166</v>
-      </c>
-      <c r="N9" s="20" t="n">
-        <v>384761041</v>
-      </c>
-      <c r="O9" s="21" t="n">
-        <v>46532432</v>
-      </c>
-      <c r="P9" s="22" t="n">
-        <v>0.120938522983152</v>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>8/9/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>125731438</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>11195807</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.08904540644798797</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>131288243</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>14045656</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>0.1069833496057983</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>25099261</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>3458247</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0.1377828215739101</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <v>48494523</v>
+      </c>
+      <c r="L9" s="18" t="n">
+        <v>4176190</v>
+      </c>
+      <c r="M9" s="19" t="n">
+        <v>0.08611673528575588</v>
+      </c>
+      <c r="N9" s="17" t="n">
+        <v>372916925</v>
+      </c>
+      <c r="O9" s="18" t="n">
+        <v>36677501</v>
+      </c>
+      <c r="P9" s="19" t="n">
+        <v>0.09835300717445312</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>+19%</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>-191bps</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>-129bps</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>+40%</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t>+366bps</t>
+        </is>
+      </c>
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>+12%</t>
+        </is>
+      </c>
+      <c r="M10" s="23" t="inlineStr">
+        <is>
+          <t>-278bps</t>
+        </is>
+      </c>
+      <c r="N10" s="21" t="inlineStr">
         <is>
           <t>+18%</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="D10" s="28" t="inlineStr">
-        <is>
-          <t>-58bps</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>+22%</t>
-        </is>
-      </c>
-      <c r="F10" s="25" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr">
-        <is>
-          <t>-163bps</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>+23%</t>
-        </is>
-      </c>
-      <c r="I10" s="29" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="J10" s="28" t="inlineStr">
-        <is>
-          <t>-559bps</t>
-        </is>
-      </c>
-      <c r="K10" s="27" t="inlineStr">
-        <is>
-          <t>-7%</t>
-        </is>
-      </c>
-      <c r="L10" s="29" t="inlineStr">
-        <is>
-          <t>-243%</t>
-        </is>
-      </c>
-      <c r="M10" s="26" t="inlineStr">
-        <is>
-          <t>+2082bps</t>
-        </is>
-      </c>
-      <c r="N10" s="24" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
       <c r="O10" s="25" t="inlineStr">
         <is>
-          <t>+28%</t>
-        </is>
-      </c>
-      <c r="P10" s="26" t="inlineStr">
-        <is>
-          <t>+140bps</t>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="P10" s="23" t="inlineStr">
+        <is>
+          <t>-121bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>7/26/2026</t>
+          <t>8/2/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>121558881</v>
+        <v>130246036</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>8980474</v>
+        <v>16204920</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.0738775639107767</v>
+        <v>0.1244177596314716</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>123109037</v>
+        <v>136855999</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>10499562</v>
+        <v>18214019</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.08528668776769004</v>
+        <v>0.133088933865442</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>24313828</v>
+        <v>33134991</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>2831499</v>
+        <v>2695236</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.1164563227147942</v>
+        <v>0.08134108139640056</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>45125668</v>
+        <v>43379501</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>2828135</v>
+        <v>5473675</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.06267242404034883</v>
+        <v>0.126181142563166</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>354055496</v>
+        <v>384761041</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>27911568</v>
+        <v>46532432</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.0788338786301456</v>
+        <v>0.120938522983152</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1373,77 +1376,77 @@
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
-          <t>+6%</t>
+          <t>+18%</t>
         </is>
       </c>
       <c r="C12" s="32" t="inlineStr">
         <is>
-          <t>-28%</t>
+          <t>+13%</t>
         </is>
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>-347bps</t>
+          <t>-58bps</t>
         </is>
       </c>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>+8%</t>
+          <t>+22%</t>
         </is>
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>-11%</t>
+          <t>+9%</t>
         </is>
       </c>
       <c r="G12" s="33" t="inlineStr">
         <is>
-          <t>-186bps</t>
+          <t>-163bps</t>
         </is>
       </c>
       <c r="H12" s="31" t="inlineStr">
         <is>
-          <t>+5%</t>
+          <t>+23%</t>
         </is>
       </c>
       <c r="I12" s="34" t="inlineStr">
         <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="J12" s="35" t="inlineStr">
-        <is>
-          <t>+76bps</t>
-        </is>
-      </c>
-      <c r="K12" s="31" t="inlineStr">
-        <is>
-          <t>+44%</t>
-        </is>
-      </c>
-      <c r="L12" s="32" t="inlineStr">
-        <is>
-          <t>-24%</t>
-        </is>
-      </c>
-      <c r="M12" s="33" t="inlineStr">
-        <is>
-          <t>-554bps</t>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>-559bps</t>
+        </is>
+      </c>
+      <c r="K12" s="35" t="inlineStr">
+        <is>
+          <t>-7%</t>
+        </is>
+      </c>
+      <c r="L12" s="34" t="inlineStr">
+        <is>
+          <t>-243%</t>
+        </is>
+      </c>
+      <c r="M12" s="36" t="inlineStr">
+        <is>
+          <t>+2082bps</t>
         </is>
       </c>
       <c r="N12" s="31" t="inlineStr">
         <is>
-          <t>+8%</t>
+          <t>+14%</t>
         </is>
       </c>
       <c r="O12" s="32" t="inlineStr">
         <is>
-          <t>-20%</t>
-        </is>
-      </c>
-      <c r="P12" s="33" t="inlineStr">
-        <is>
-          <t>-273bps</t>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="P12" s="36" t="inlineStr">
+        <is>
+          <t>+140bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Wed Sep  9 21:27:44 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,6 +210,15 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -231,49 +240,37 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -783,53 +780,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>8/30/2026</t>
+          <t>9/6/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>149527600</v>
+        <v>171492780</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>12079306</v>
+        <v>16692306</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.08078311963811363</v>
+        <v>0.0973353280528778</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>146777769</v>
+        <v>167953524</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>15874317</v>
+        <v>16892923</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.1081520526449751</v>
+        <v>0.1005809380933263</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>29155390</v>
+        <v>34668902</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>2727869</v>
+        <v>3546293</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.09356311131492324</v>
+        <v>0.1022903177031681</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>52848942</v>
+        <v>56782523</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>5061346</v>
+        <v>3258000</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.09577005344780601</v>
+        <v>0.05737680941017714</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>420285714</v>
+        <v>483313174</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>39300665</v>
+        <v>44849147</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.09350940013154956</v>
+        <v>0.09279520901286253</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -840,264 +837,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>-10%</t>
+          <t>-16%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>-39%</t>
+          <t>+273%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>-392bps</t>
+          <t>+756bps</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>-4%</t>
+          <t>-3%</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>-27%</t>
+          <t>+16%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>-338bps</t>
+          <t>+168bps</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>-25%</t>
+          <t>-6%</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>-37%</t>
+          <t>+87%</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>-186bps</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>-64%</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>-66%</t>
-        </is>
-      </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>-57bps</t>
+          <t>+509bps</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>-45%</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>-567bps</t>
         </is>
       </c>
       <c r="N4" s="13" t="inlineStr">
         <is>
-          <t>-25%</t>
+          <t>-8%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>-41%</t>
+          <t>+47%</t>
         </is>
       </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
-          <t>-259bps</t>
+          <t>+349bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>8/23/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="n">
-        <v>137507207</v>
-      </c>
-      <c r="C5" s="18" t="n">
-        <v>10643451</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>0.07740285932794781</v>
-      </c>
-      <c r="E5" s="17" t="n">
-        <v>132060011</v>
-      </c>
-      <c r="F5" s="18" t="n">
-        <v>10710519</v>
-      </c>
-      <c r="G5" s="19" t="n">
-        <v>0.08110342350342527</v>
-      </c>
-      <c r="H5" s="17" t="n">
-        <v>24881322</v>
-      </c>
-      <c r="I5" s="18" t="n">
-        <v>1911178</v>
-      </c>
-      <c r="J5" s="19" t="n">
-        <v>0.07681175461657544</v>
-      </c>
-      <c r="K5" s="17" t="n">
-        <v>47701558</v>
-      </c>
-      <c r="L5" s="18" t="n">
-        <v>3476356</v>
-      </c>
-      <c r="M5" s="19" t="n">
-        <v>0.07287720036314117</v>
-      </c>
-      <c r="N5" s="17" t="n">
-        <v>381646903</v>
-      </c>
-      <c r="O5" s="18" t="n">
-        <v>30506351</v>
-      </c>
-      <c r="P5" s="19" t="n">
-        <v>0.07993344308626553</v>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>8/30/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>149527600</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>12079306</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>0.08078311963811363</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>146777769</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>15874317</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.1081520526449751</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>29155390</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>2727869</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.09356311131492324</v>
+      </c>
+      <c r="K5" s="20" t="n">
+        <v>52848942</v>
+      </c>
+      <c r="L5" s="21" t="n">
+        <v>5061346</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.09577005344780601</v>
+      </c>
+      <c r="N5" s="20" t="n">
+        <v>420285714</v>
+      </c>
+      <c r="O5" s="21" t="n">
+        <v>39300665</v>
+      </c>
+      <c r="P5" s="22" t="n">
+        <v>0.09350940013154956</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>+4%</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="inlineStr">
-        <is>
-          <t>-31%</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>-395bps</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>-10%</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>-39%</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>-392bps</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>-4%</t>
         </is>
       </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>-78bps</t>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>-338bps</t>
         </is>
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="I6" s="22" t="inlineStr">
-        <is>
-          <t>-36%</t>
-        </is>
-      </c>
-      <c r="J6" s="23" t="inlineStr">
-        <is>
-          <t>-301bps</t>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>-37%</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>-186bps</t>
         </is>
       </c>
       <c r="K6" s="24" t="inlineStr">
         <is>
-          <t>-78%</t>
+          <t>-64%</t>
         </is>
       </c>
       <c r="L6" s="25" t="inlineStr">
         <is>
-          <t>+688%</t>
+          <t>-66%</t>
         </is>
       </c>
       <c r="M6" s="26" t="inlineStr">
         <is>
-          <t>+708bps</t>
+          <t>-57bps</t>
         </is>
       </c>
       <c r="N6" s="24" t="inlineStr">
         <is>
-          <t>-30%</t>
-        </is>
-      </c>
-      <c r="O6" s="22" t="inlineStr">
-        <is>
-          <t>-11%</t>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="O6" s="25" t="inlineStr">
+        <is>
+          <t>-41%</t>
         </is>
       </c>
       <c r="P6" s="26" t="inlineStr">
         <is>
-          <t>+170bps</t>
+          <t>-259bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>8/16/2026</t>
+          <t>8/23/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>139804782</v>
+        <v>137507207</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>14936414</v>
+        <v>10643451</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.1068376473703167</v>
+        <v>0.07740285932794781</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>128334482</v>
+        <v>132060011</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>16567440</v>
+        <v>10710519</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1290957795738794</v>
+        <v>0.08110342350342527</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>26211607</v>
+        <v>24881322</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>3989974</v>
+        <v>1911178</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.1522216474556482</v>
+        <v>0.07681175461657544</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>43618315</v>
+        <v>47701558</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>4332991</v>
+        <v>3476356</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.09933879839237256</v>
+        <v>0.07287720036314117</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>380789208</v>
+        <v>381646903</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>44525193</v>
+        <v>30506351</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.1169287155848177</v>
+        <v>0.07993344308626553</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1106,266 +1103,266 @@
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>+182bps</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="F8" s="28" t="inlineStr">
-        <is>
-          <t>+17%</t>
-        </is>
-      </c>
-      <c r="G8" s="29" t="inlineStr">
-        <is>
-          <t>+80bps</t>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>-31%</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>-395bps</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>-78bps</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>-1%</t>
-        </is>
-      </c>
-      <c r="I8" s="28" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="J8" s="29" t="inlineStr">
-        <is>
-          <t>+590bps</t>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>-36%</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>-301bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>-70%</t>
-        </is>
-      </c>
-      <c r="L8" s="28" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="M8" s="29" t="inlineStr">
-        <is>
-          <t>+811bps</t>
+          <t>-78%</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>+688%</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>+708bps</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>-17%</t>
-        </is>
-      </c>
-      <c r="O8" s="28" t="inlineStr">
-        <is>
-          <t>+34%</t>
-        </is>
-      </c>
-      <c r="P8" s="29" t="inlineStr">
-        <is>
-          <t>+441bps</t>
+          <t>-30%</t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="P8" s="15" t="inlineStr">
+        <is>
+          <t>+170bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>8/9/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="n">
-        <v>125731438</v>
-      </c>
-      <c r="C9" s="18" t="n">
-        <v>11195807</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>0.08904540644798797</v>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>131288243</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>14045656</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>0.1069833496057983</v>
-      </c>
-      <c r="H9" s="17" t="n">
-        <v>25099261</v>
-      </c>
-      <c r="I9" s="18" t="n">
-        <v>3458247</v>
-      </c>
-      <c r="J9" s="19" t="n">
-        <v>0.1377828215739101</v>
-      </c>
-      <c r="K9" s="17" t="n">
-        <v>48494523</v>
-      </c>
-      <c r="L9" s="18" t="n">
-        <v>4176190</v>
-      </c>
-      <c r="M9" s="19" t="n">
-        <v>0.08611673528575588</v>
-      </c>
-      <c r="N9" s="17" t="n">
-        <v>372916925</v>
-      </c>
-      <c r="O9" s="18" t="n">
-        <v>36677501</v>
-      </c>
-      <c r="P9" s="19" t="n">
-        <v>0.09835300717445312</v>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>8/16/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>139804782</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>14936414</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.1068376473703167</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>128334482</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>16567440</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>0.1290957795738794</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>26211607</v>
+      </c>
+      <c r="I9" s="21" t="n">
+        <v>3989974</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.1522216474556482</v>
+      </c>
+      <c r="K9" s="20" t="n">
+        <v>43618315</v>
+      </c>
+      <c r="L9" s="21" t="n">
+        <v>4332991</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>0.09933879839237256</v>
+      </c>
+      <c r="N9" s="20" t="n">
+        <v>380789208</v>
+      </c>
+      <c r="O9" s="21" t="n">
+        <v>44525193</v>
+      </c>
+      <c r="P9" s="22" t="n">
+        <v>0.1169287155848177</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>+19%</t>
-        </is>
-      </c>
-      <c r="C10" s="22" t="inlineStr">
-        <is>
-          <t>-2%</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>-191bps</t>
-        </is>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
-          <t>+16%</t>
-        </is>
-      </c>
-      <c r="F10" s="25" t="inlineStr">
-        <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>-129bps</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="inlineStr">
-        <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="I10" s="25" t="inlineStr">
-        <is>
-          <t>+40%</t>
-        </is>
-      </c>
-      <c r="J10" s="26" t="inlineStr">
-        <is>
-          <t>+366bps</t>
-        </is>
-      </c>
-      <c r="K10" s="21" t="inlineStr">
-        <is>
-          <t>+48%</t>
-        </is>
-      </c>
-      <c r="L10" s="25" t="inlineStr">
-        <is>
-          <t>+12%</t>
-        </is>
-      </c>
-      <c r="M10" s="23" t="inlineStr">
-        <is>
-          <t>-278bps</t>
-        </is>
-      </c>
-      <c r="N10" s="21" t="inlineStr">
-        <is>
-          <t>+18%</t>
-        </is>
-      </c>
-      <c r="O10" s="25" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="P10" s="23" t="inlineStr">
-        <is>
-          <t>-121bps</t>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>+14%</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>+182bps</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>+17%</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>+80bps</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>-1%</t>
+        </is>
+      </c>
+      <c r="I10" s="28" t="inlineStr">
+        <is>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>+590bps</t>
+        </is>
+      </c>
+      <c r="K10" s="24" t="inlineStr">
+        <is>
+          <t>-70%</t>
+        </is>
+      </c>
+      <c r="L10" s="28" t="inlineStr">
+        <is>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="M10" s="29" t="inlineStr">
+        <is>
+          <t>+811bps</t>
+        </is>
+      </c>
+      <c r="N10" s="24" t="inlineStr">
+        <is>
+          <t>-17%</t>
+        </is>
+      </c>
+      <c r="O10" s="28" t="inlineStr">
+        <is>
+          <t>+34%</t>
+        </is>
+      </c>
+      <c r="P10" s="29" t="inlineStr">
+        <is>
+          <t>+441bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>8/2/2026</t>
+          <t>8/9/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>130246036</v>
+        <v>125731438</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>16204920</v>
+        <v>11195807</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.1244177596314716</v>
+        <v>0.08904540644798797</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>136855999</v>
+        <v>131288243</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>18214019</v>
+        <v>14045656</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.133088933865442</v>
+        <v>0.1069833496057983</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>33134991</v>
+        <v>25099261</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>2695236</v>
+        <v>3458247</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.08134108139640056</v>
+        <v>0.1377828215739101</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>43379501</v>
+        <v>48494523</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>5473675</v>
+        <v>4176190</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.126181142563166</v>
+        <v>0.08611673528575588</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>384761041</v>
+        <v>372916925</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>46532432</v>
+        <v>36677501</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.120938522983152</v>
+        <v>0.09835300717445312</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1376,77 +1373,77 @@
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
+          <t>+19%</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>-191bps</t>
+        </is>
+      </c>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>-129bps</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="I12" s="34" t="inlineStr">
+        <is>
+          <t>+40%</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>+366bps</t>
+        </is>
+      </c>
+      <c r="K12" s="31" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
+      <c r="L12" s="34" t="inlineStr">
+        <is>
+          <t>+12%</t>
+        </is>
+      </c>
+      <c r="M12" s="33" t="inlineStr">
+        <is>
+          <t>-278bps</t>
+        </is>
+      </c>
+      <c r="N12" s="31" t="inlineStr">
+        <is>
           <t>+18%</t>
         </is>
       </c>
-      <c r="C12" s="32" t="inlineStr">
-        <is>
-          <t>+13%</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>-58bps</t>
-        </is>
-      </c>
-      <c r="E12" s="31" t="inlineStr">
-        <is>
-          <t>+22%</t>
-        </is>
-      </c>
-      <c r="F12" s="32" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="G12" s="33" t="inlineStr">
-        <is>
-          <t>-163bps</t>
-        </is>
-      </c>
-      <c r="H12" s="31" t="inlineStr">
-        <is>
-          <t>+23%</t>
-        </is>
-      </c>
-      <c r="I12" s="34" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="J12" s="33" t="inlineStr">
-        <is>
-          <t>-559bps</t>
-        </is>
-      </c>
-      <c r="K12" s="35" t="inlineStr">
-        <is>
-          <t>-7%</t>
-        </is>
-      </c>
-      <c r="L12" s="34" t="inlineStr">
-        <is>
-          <t>-243%</t>
-        </is>
-      </c>
-      <c r="M12" s="36" t="inlineStr">
-        <is>
-          <t>+2082bps</t>
-        </is>
-      </c>
-      <c r="N12" s="31" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="O12" s="32" t="inlineStr">
-        <is>
-          <t>+28%</t>
-        </is>
-      </c>
-      <c r="P12" s="36" t="inlineStr">
-        <is>
-          <t>+140bps</t>
+      <c r="O12" s="34" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="P12" s="33" t="inlineStr">
+        <is>
+          <t>-121bps</t>
         </is>
       </c>
     </row>

</xml_diff>